<commit_message>
Final-Cleanup: OUT_DIR + Workflow-Pfade + Excel-Hyperlinks
- generate.py OUT_DIR default v2/ → code/ (Repo-Refactor v2 → code)
- q-end-routine.yml Methodik-Pfad pm-dashboards/v2/METHODE.md → code/METHODE.md
- Excel Anleitung Q-Wechsel: Hyperlinks zu ANLEITUNG_QUARTALSWECHSEL.md + METHODE.md

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="179" formatCode="#,##0.0"/>
     <numFmt numFmtId="180" formatCode="#,##0 €"/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -358,6 +358,14 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
+    <font>
+      <color rgb="000066CC"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="34">
@@ -664,7 +672,7 @@
     <xf numFmtId="43" fontId="24" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1076,6 +1084,8 @@
     <xf numFmtId="180" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="180" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1578,6 +1588,30 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="169" t="inlineStr">
+        <is>
+          <t>Vollständige Anleitung:</t>
+        </is>
+      </c>
+      <c r="B18" s="170" t="inlineStr">
+        <is>
+          <t>github.com/virmen/vacura-pm-dash-9f3k2/blob/main/ANLEITUNG_QUARTALSWECHSEL.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="169" t="inlineStr">
+        <is>
+          <t>Berechnungs-Methodik:</t>
+        </is>
+      </c>
+      <c r="B19" s="170" t="inlineStr">
+        <is>
+          <t>github.com/virmen/vacura-pm-dash-9f3k2/blob/main/METHODE.md</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="138" t="inlineStr">
         <is>
@@ -1598,6 +1632,10 @@
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1895,8 +1933,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A12:J12"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A12:J12"/>
     <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Q-End-Routine: auto automatisch befüllt (2026-07-08T05:59Z)
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6700" yWindow="-19780" windowWidth="24200" windowHeight="15120" tabRatio="500" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modell" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Modell" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1646,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="97" min="1" max="1"/>
@@ -1896,6 +1896,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="162" t="inlineStr">
         <is>
@@ -1931,11 +1932,45 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1947,7 +1982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="97" min="1" max="1"/>
@@ -2413,6 +2448,390 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Laura</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>5198.4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>721</v>
+      </c>
+      <c r="J16" t="n">
+        <v>343.5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>265339</v>
+      </c>
+      <c r="L16" t="n">
+        <v>4133.9</v>
+      </c>
+      <c r="M16" t="n">
+        <v>64.19</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏳ Zufriedenheit fehlt</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2026-07-08 05:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Marleen</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>7528.9</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1346.5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>440.5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>371864</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5741.9</v>
+      </c>
+      <c r="M17" t="n">
+        <v>64.76000000000001</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>⏳ Zufriedenheit fehlt</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-07-08 05:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Luise</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>7528.9</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1346.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>440.5</v>
+      </c>
+      <c r="K18" t="n">
+        <v>371864</v>
+      </c>
+      <c r="L18" t="n">
+        <v>5741.9</v>
+      </c>
+      <c r="M18" t="n">
+        <v>64.76000000000001</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>⏳ Zufriedenheit fehlt</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2026-07-08 05:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>5198.4</v>
+      </c>
+      <c r="I19" t="n">
+        <v>721</v>
+      </c>
+      <c r="J19" t="n">
+        <v>343.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>265339</v>
+      </c>
+      <c r="L19" t="n">
+        <v>4133.9</v>
+      </c>
+      <c r="M19" t="n">
+        <v>64.19</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>⏳ Zufriedenheit fehlt</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>2026-07-08 05:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2531,7 +2950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="97" min="1" max="1"/>
@@ -2654,6 +3073,8 @@
         <v>89.48</v>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="113" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Emily als 5. PM angelegt + Q-Label-Fix in Q-End-Routine
- PM-Stammdaten: Emily (40h, Bundle FH/CB/PB, Start 01.07.2026), Token auto-erzeugt
- Marleen/Luise: PM-Std Bundle 80 → 120, Bundle-PMs um Emily ergänzt; Max 26h → 30h
- Q-End-Routine normalisiert Quartals-Label auf Sheet-Format ('Q2 2026' statt '2026-Q2')
  — behebt die Duplikat-Zeilen vom Lauf am 08.07.; '2026-Q2'-Zeilen entfernt
- Dashboards mit neuem Bundle-Split regeneriert

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6700" yWindow="-19780" windowWidth="24200" windowHeight="15120" tabRatio="500" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4600" yWindow="-19780" windowWidth="24200" windowHeight="15120" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Modell" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modell" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -21,26 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="17">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0&quot; h&quot;"/>
-    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="170" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    <numFmt numFmtId="171" formatCode="#,##0&quot; h&quot;"/>
-    <numFmt numFmtId="172" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="174" formatCode="#,##0.00&quot; €&quot;"/>
-    <numFmt numFmtId="175" formatCode="0&quot; h&quot;"/>
-    <numFmt numFmtId="176" formatCode="#,##0.00&quot; €/h&quot;"/>
-    <numFmt numFmtId="177" formatCode="\+#,##0&quot; €&quot;"/>
-    <numFmt numFmtId="178" formatCode="\+#,##0.00&quot; €/h&quot;"/>
-    <numFmt numFmtId="179" formatCode="#,##0.0"/>
-    <numFmt numFmtId="180" formatCode="#,##0 €"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0\ \€"/>
   </numFmts>
-  <fonts count="55">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -95,110 +83,7 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF333333"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF333333"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF333333"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color rgb="FF37474F"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color rgb="FF666666"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -269,20 +154,42 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
+      <color rgb="FF1A8A8B"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF263238"/>
-      <sz val="18"/>
+      <i val="1"/>
+      <color rgb="FF666666"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -294,81 +201,19 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF1B5E20"/>
+      <color rgb="FF0066CC"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-    </font>
-    <font>
-      <name val="SF Mono"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001A8A8B"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-    </font>
-    <font>
-      <color rgb="000066CC"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -385,76 +230,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFDE9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF263238"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF607D8B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF455A64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFECEFF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF8E1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4EC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFECB3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC8E6C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB71C1C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF263238"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF455A64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFECEFF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -494,51 +269,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFECB3"/>
+        <fgColor rgb="FF1A8A8B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF455A64"/>
+        <fgColor rgb="FFFFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE0F2F1"/>
+        <fgColor rgb="FFD4EDDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A8A8B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F4F4"/>
+        <fgColor rgb="FFE8F4F4"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -576,103 +326,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF455A64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF455A64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="24" fillId="0" borderId="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -700,397 +358,109 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="12" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="171" fontId="23" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="28" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="175" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="37" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="37" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="36" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="36" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="35" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="41" fillId="26" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="42" fillId="27" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="42" fillId="27" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="39" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="24" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="37" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="36" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="36" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="25" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="35" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="23" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="28" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="46" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="45" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="47" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Komma" xfId="1" builtinId="3"/>
-    <cellStyle name="Währung" xfId="2" builtinId="4"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1348,272 +718,272 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="97" min="1" max="1"/>
-    <col width="40" customWidth="1" style="97" min="2" max="2"/>
-    <col width="35" customWidth="1" style="97" min="3" max="3"/>
-    <col width="22" customWidth="1" style="97" min="4" max="4"/>
-    <col width="60" customWidth="1" style="97" min="5" max="5"/>
+    <col width="8" customWidth="1" style="44" min="1" max="1"/>
+    <col width="40" customWidth="1" style="44" min="2" max="2"/>
+    <col width="35" customWidth="1" style="44" min="3" max="3"/>
+    <col width="22" customWidth="1" style="44" min="4" max="4"/>
+    <col width="60" customWidth="1" style="44" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="136" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="44">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>📋 Anleitung Quartalswechsel — Was tun, wenn ein Quartal endet?</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="97">
-      <c r="A3" s="137" t="inlineStr">
+    <row r="3" ht="30" customHeight="1" s="44">
+      <c r="A3" s="55" t="inlineStr">
         <is>
           <t>Diese Anleitung beschreibt die manuellen Schritte, die nach jedem Quartals-Ende notwendig sind, damit die PM-Bewertung für das Folge-Quartal greift.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="138" t="inlineStr">
+    <row r="5" ht="16" customHeight="1" s="44">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Zeitpunkt: spätestens 5. Tag des Folge-Monats (also 5.7., 5.10., 5.1., 5.4.)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="139" t="inlineStr">
+    <row r="7" ht="16" customHeight="1" s="44">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Schritt</t>
         </is>
       </c>
-      <c r="B7" s="139" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>Was</t>
         </is>
       </c>
-      <c r="C7" s="139" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>Wo eintragen</t>
         </is>
       </c>
-      <c r="D7" s="139" t="inlineStr">
+      <c r="D7" s="28" t="inlineStr">
         <is>
           <t>Wer</t>
         </is>
       </c>
-      <c r="E7" s="139" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>Warum / Hinweis</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="75" customHeight="1" s="97">
-      <c r="A8" s="140" t="inlineStr">
+    <row r="8" ht="75" customHeight="1" s="44">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B8" s="141" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Zufriedenheits-Scores aus Q-Umfrage eintragen</t>
         </is>
       </c>
-      <c r="C8" s="141" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>Tab "Daten" — Spalten 11 (Rücken), 12 (Komm), 13 (eNPS)</t>
         </is>
       </c>
-      <c r="D8" s="141" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Du (Geschäftsführung)</t>
         </is>
       </c>
-      <c r="E8" s="141" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>Aus quartalsweiser Umfrage (anonym, ≥60% Teilnahme). Formel: Score = 0,2×Rücken + 0,2×Komm + 0,6×eNPS. Ohne diese Werte ist die Stufen-Bewertung unvollständig.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="75" customHeight="1" s="97">
-      <c r="A9" s="140" t="inlineStr">
+    <row r="9" ht="75" customHeight="1" s="44">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B9" s="141" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>MediFox-IST-Werte als Sanity-Check eintragen</t>
         </is>
       </c>
-      <c r="C9" s="141" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>Tab "Sanity (MediFox)" — pro Bundle eine Zeile</t>
         </is>
       </c>
-      <c r="D9" s="141" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Du (Geschäftsführung)</t>
         </is>
       </c>
-      <c r="E9" s="141" t="inlineStr">
+      <c r="E9" s="30" t="inlineStr">
         <is>
           <t>MediFox-Export pro Standort/Monat, Summen über Q. Wird automatisch mit NocoDB-IST verglichen — Diff &gt; 2 % bedeutet Untersuchung nötig.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="75" customHeight="1" s="97">
-      <c r="A10" s="142" t="inlineStr">
+    <row r="10" ht="75" customHeight="1" s="44">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B10" s="143" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>Q-End-Berechnung anstoßen</t>
         </is>
       </c>
-      <c r="C10" s="143" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>Routine läuft automatisch am 1. des Folge-Monats</t>
         </is>
       </c>
-      <c r="D10" s="143" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>Code (Routine-Agent)</t>
         </is>
       </c>
-      <c r="E10" s="143" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>compute_quartal() rechnet für jedes Bundle: IST, Vstd, Abw, Feiertage, eur60, rechn_stufe und tats_stufe (mit ±1-Deckel). Werte werden ins Tab "Audit Q&lt;N&gt;" geschrieben.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="75" customHeight="1" s="97">
-      <c r="A11" s="140" t="inlineStr">
+    <row r="11" ht="75" customHeight="1" s="44">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B11" s="141" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Stufe Vorquartal manuell updaten</t>
         </is>
       </c>
-      <c r="C11" s="141" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>Tab "Daten" — Spalte 5 ("Stufe Vorquartal") pro PM</t>
         </is>
       </c>
-      <c r="D11" s="141" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>Du (Geschäftsführung) ODER Routine</t>
         </is>
       </c>
-      <c r="E11" s="141" t="inlineStr">
+      <c r="E11" s="30" t="inlineStr">
         <is>
           <t>Die tats_stufe aus dem Audit-Tab wird zur "Stufe Vorquartal" für die nächste Bewertung — wichtig für den ±1-Deckel. Wenn falsch, kann eine PM rechnerisch Stufe 4 sein aber wegen falschem Vorquartals-Wert auf Stufe 1 gedeckelt werden.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="75" customHeight="1" s="97">
-      <c r="A12" s="142" t="inlineStr">
+    <row r="12" ht="75" customHeight="1" s="44">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B12" s="143" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>Dashboards regenerieren + deployen</t>
         </is>
       </c>
-      <c r="C12" s="143" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>GitHub Action "Regenerate PM Dashboards" manuell triggern</t>
         </is>
       </c>
-      <c r="D12" s="143" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>Code (Routine-Agent)</t>
         </is>
       </c>
-      <c r="E12" s="143" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>Nach Excel-Update werden die HTML-Dashboards mit Q-Final-Werten neu gebaut und auf GitHub Pages deployed. PMs sehen dann ihre offizielle Q-Bewertung.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="75" customHeight="1" s="97">
-      <c r="A13" s="140" t="inlineStr">
+    <row r="13" ht="75" customHeight="1" s="44">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B13" s="141" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>Plausibilitäts-Check + Freigabe</t>
         </is>
       </c>
-      <c r="C13" s="141" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>Audit-Tab durchgehen, Diff zu MediFox prüfen</t>
         </is>
       </c>
-      <c r="D13" s="141" t="inlineStr">
+      <c r="D13" s="30" t="inlineStr">
         <is>
           <t>Du (Geschäftsführung)</t>
         </is>
       </c>
-      <c r="E13" s="141" t="inlineStr">
+      <c r="E13" s="30" t="inlineStr">
         <is>
           <t>Wenn Audit-Werte plausibel und MediFox-Diff &lt; 2 %: Q-Bewertung gilt als final, Gehälter werden für das Folge-Quartal angepasst. Sonst: Ursache klären, Werte ggf. nachbessern.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="138" t="inlineStr">
+    <row r="15" ht="16" customHeight="1" s="44">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>Legende:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="144" t="inlineStr">
+      <c r="A16" s="51" t="inlineStr">
         <is>
           <t>Gelb = manuelle Aktion durch Geschäftsführung</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="145" t="inlineStr">
+      <c r="A17" s="54" t="inlineStr">
         <is>
           <t>Grün = automatisch durch Code/Routine</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="169" t="inlineStr">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Vollständige Anleitung:</t>
         </is>
       </c>
-      <c r="B18" s="170" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr">
         <is>
           <t>github.com/virmen/vacura-pm-dash-9f3k2/blob/main/ANLEITUNG_QUARTALSWECHSEL.md</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="169" t="inlineStr">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>Berechnungs-Methodik:</t>
         </is>
       </c>
-      <c r="B19" s="170" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>github.com/virmen/vacura-pm-dash-9f3k2/blob/main/METHODE.md</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="138" t="inlineStr">
+    <row r="20" ht="16" customHeight="1" s="44">
+      <c r="A20" s="53" t="inlineStr">
         <is>
           <t>Detaillierte Berechnungsmethodik</t>
         </is>
@@ -1647,292 +1017,331 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="97" min="1" max="1"/>
-    <col width="10" customWidth="1" style="97" min="2" max="2"/>
-    <col width="12" customWidth="1" style="97" min="3" max="3"/>
-    <col width="12" customWidth="1" style="97" min="4" max="4"/>
-    <col width="14" customWidth="1" style="97" min="5" max="5"/>
-    <col width="35" customWidth="1" style="97" min="6" max="6"/>
-    <col width="18" customWidth="1" style="97" min="7" max="7"/>
-    <col width="12" customWidth="1" style="97" min="8" max="8"/>
-    <col width="35" customWidth="1" style="97" min="9" max="9"/>
-    <col width="8" customWidth="1" style="97" min="10" max="10"/>
+    <col width="10" customWidth="1" style="44" min="1" max="2"/>
+    <col width="12" customWidth="1" style="44" min="3" max="4"/>
+    <col width="14" customWidth="1" style="44" min="5" max="5"/>
+    <col width="35" customWidth="1" style="44" min="6" max="6"/>
+    <col width="18" customWidth="1" style="44" min="7" max="7"/>
+    <col width="12" customWidth="1" style="44" min="8" max="8"/>
+    <col width="35" customWidth="1" style="44" min="9" max="9"/>
+    <col width="8" customWidth="1" style="44" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="136" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="44">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>👥 PM-Stammdaten (Quelle der Wahrheit für PM-Liste)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="97">
-      <c r="A3" s="137" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="44">
+      <c r="A3" s="55" t="inlineStr">
         <is>
           <t>Quelle der Wahrheit für die PM-Liste. Code liest beim Start automatisch.
 ➜ Neuen PM anlegen: einfach neue Zeile anhängen. Spalte 8 (Farbe), 9 (Token) und 10 (Aktiv) dürfen leer bleiben — werden beim nächsten Dashboard-Lauf automatisch befüllt. Token wird automatisch erzeugt und ins Excel zurückgeschrieben.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="97">
-      <c r="A5" s="147" t="inlineStr">
+    <row r="5" ht="30" customHeight="1" s="44">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B5" s="147" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>Wochenstd</t>
         </is>
       </c>
-      <c r="C5" s="147" t="inlineStr">
+      <c r="C5" s="34" t="inlineStr">
         <is>
           <t>PM-Std Bundle</t>
         </is>
       </c>
-      <c r="D5" s="147" t="inlineStr">
+      <c r="D5" s="34" t="inlineStr">
         <is>
           <t>Mindestgehalt</t>
         </is>
       </c>
-      <c r="E5" s="147" t="inlineStr">
+      <c r="E5" s="34" t="inlineStr">
         <is>
           <t>Startdatum</t>
         </is>
       </c>
-      <c r="F5" s="147" t="inlineStr">
+      <c r="F5" s="34" t="inlineStr">
         <is>
           <t>Bundle-Standorte</t>
         </is>
       </c>
-      <c r="G5" s="147" t="inlineStr">
+      <c r="G5" s="34" t="inlineStr">
         <is>
           <t>Bundle-PMs</t>
         </is>
       </c>
-      <c r="H5" s="147" t="inlineStr">
+      <c r="H5" s="34" t="inlineStr">
         <is>
           <t>Farbe (Hex)</t>
         </is>
       </c>
-      <c r="I5" s="147" t="inlineStr">
+      <c r="I5" s="34" t="inlineStr">
         <is>
           <t>URL-Token (32-hex)</t>
         </is>
       </c>
-      <c r="J5" s="147" t="inlineStr">
+      <c r="J5" s="34" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="137" t="inlineStr">
+    <row r="6" ht="16" customHeight="1" s="44">
+      <c r="A6" s="55" t="inlineStr">
         <is>
           <t>Laura</t>
         </is>
       </c>
-      <c r="B6" s="137" t="n">
+      <c r="B6" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="C6" s="137" t="n">
+      <c r="C6" s="55" t="n">
         <v>65</v>
       </c>
-      <c r="D6" s="137" t="n">
+      <c r="D6" s="55" t="n">
         <v>45000</v>
       </c>
-      <c r="E6" s="137" t="n"/>
-      <c r="F6" s="137" t="inlineStr">
+      <c r="E6" s="55" t="n"/>
+      <c r="F6" s="55" t="inlineStr">
         <is>
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="G6" s="137" t="inlineStr">
+      <c r="G6" s="55" t="inlineStr">
         <is>
           <t>Laura, Max</t>
         </is>
       </c>
-      <c r="H6" s="137" t="inlineStr">
+      <c r="H6" s="55" t="inlineStr">
         <is>
           <t>#4CAF50</t>
         </is>
       </c>
-      <c r="I6" s="137" t="inlineStr">
+      <c r="I6" s="55" t="inlineStr">
         <is>
           <t>8278b207ba9e80605ae5f1604d696759</t>
         </is>
       </c>
-      <c r="J6" s="137" t="b">
+      <c r="J6" s="55" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="137" t="inlineStr">
+    <row r="7" ht="32" customHeight="1" s="44">
+      <c r="A7" s="55" t="inlineStr">
         <is>
           <t>Marleen</t>
         </is>
       </c>
-      <c r="B7" s="137" t="n">
+      <c r="B7" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="C7" s="137" t="n">
-        <v>80</v>
-      </c>
-      <c r="D7" s="137" t="n">
+      <c r="C7" s="55" t="n">
+        <v>120</v>
+      </c>
+      <c r="D7" s="55" t="n">
         <v>45000</v>
       </c>
-      <c r="E7" s="137" t="n"/>
-      <c r="F7" s="137" t="inlineStr">
+      <c r="E7" s="55" t="n"/>
+      <c r="F7" s="55" t="inlineStr">
         <is>
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="G7" s="137" t="inlineStr">
-        <is>
-          <t>Marleen, Luise</t>
-        </is>
-      </c>
-      <c r="H7" s="137" t="inlineStr">
+      <c r="G7" s="55" t="inlineStr">
+        <is>
+          <t>Marleen, Luise, Emily</t>
+        </is>
+      </c>
+      <c r="H7" s="55" t="inlineStr">
         <is>
           <t>#2196F3</t>
         </is>
       </c>
-      <c r="I7" s="137" t="inlineStr">
+      <c r="I7" s="55" t="inlineStr">
         <is>
           <t>0093979f8cf4df0f67ec20b6e35e6beb</t>
         </is>
       </c>
-      <c r="J7" s="137" t="b">
+      <c r="J7" s="55" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="137" t="inlineStr">
+    <row r="8" ht="32" customHeight="1" s="44">
+      <c r="A8" s="55" t="inlineStr">
         <is>
           <t>Luise</t>
         </is>
       </c>
-      <c r="B8" s="137" t="n">
+      <c r="B8" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="137" t="n">
-        <v>80</v>
-      </c>
-      <c r="D8" s="137" t="n">
+      <c r="C8" s="55" t="n">
+        <v>120</v>
+      </c>
+      <c r="D8" s="55" t="n">
         <v>40000</v>
       </c>
-      <c r="E8" s="137" t="inlineStr">
+      <c r="E8" s="55" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="F8" s="137" t="inlineStr">
+      <c r="F8" s="55" t="inlineStr">
         <is>
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="G8" s="137" t="inlineStr">
-        <is>
-          <t>Marleen, Luise</t>
-        </is>
-      </c>
-      <c r="H8" s="137" t="inlineStr">
+      <c r="G8" s="55" t="inlineStr">
+        <is>
+          <t>Marleen, Luise, Emily</t>
+        </is>
+      </c>
+      <c r="H8" s="55" t="inlineStr">
         <is>
           <t>#9C27B0</t>
         </is>
       </c>
-      <c r="I8" s="137" t="inlineStr">
+      <c r="I8" s="55" t="inlineStr">
         <is>
           <t>52981192518b734a346928ed713bc015</t>
         </is>
       </c>
-      <c r="J8" s="137" t="b">
+      <c r="J8" s="55" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="137" t="inlineStr">
+    <row r="9" ht="16" customHeight="1" s="44">
+      <c r="A9" s="55" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="B9" s="137" t="n">
-        <v>26</v>
-      </c>
-      <c r="C9" s="137" t="n">
+      <c r="B9" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="C9" s="55" t="n">
         <v>65</v>
       </c>
-      <c r="D9" s="137" t="n">
+      <c r="D9" s="55" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="137" t="inlineStr">
+      <c r="E9" s="55" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="F9" s="137" t="inlineStr">
+      <c r="F9" s="55" t="inlineStr">
         <is>
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="G9" s="137" t="inlineStr">
+      <c r="G9" s="55" t="inlineStr">
         <is>
           <t>Laura, Max</t>
         </is>
       </c>
-      <c r="H9" s="137" t="inlineStr">
+      <c r="H9" s="55" t="inlineStr">
         <is>
           <t>#FF9800</t>
         </is>
       </c>
-      <c r="I9" s="137" t="inlineStr">
+      <c r="I9" s="55" t="inlineStr">
         <is>
           <t>5051837ce5b8f243f109306f60136f17</t>
         </is>
       </c>
-      <c r="J9" s="137" t="b">
+      <c r="J9" s="55" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="162" t="inlineStr">
+    <row r="10" ht="32" customHeight="1" s="44">
+      <c r="A10" s="55" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>40</v>
+      </c>
+      <c r="C10" s="55" t="n">
+        <v>120</v>
+      </c>
+      <c r="D10" s="55" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E10" s="59" t="n">
+        <v>46204</v>
+      </c>
+      <c r="F10" s="55" t="inlineStr">
+        <is>
+          <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
+        </is>
+      </c>
+      <c r="G10" s="55" t="inlineStr">
+        <is>
+          <t>Marleen, Luise, Emily</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>#0D595A</t>
+        </is>
+      </c>
+      <c r="I10" s="55" t="inlineStr">
+        <is>
+          <t>34ff01c507e5f18ac55f03759f68f856</t>
+        </is>
+      </c>
+      <c r="J10" s="55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Auto-Befüllung beim Dashboard-Lauf:</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="163" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="56" t="inlineStr">
         <is>
           <t>• Spalte 8 leer → Default-Farbe #0D595A (Vacura-Teal)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="163" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>• Spalte 9 leer → Token wird per secrets.token_hex(16) erzeugt + hier eingetragen</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="163" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="56" t="inlineStr">
         <is>
           <t>• Spalte 10 leer → Aktiv=Ja angenommen. Auf FALSE setzen um PM zu deaktivieren (z.B. Austritt)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="163" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="56" t="inlineStr">
         <is>
           <t>• Plus: Daten-Tab Stammdaten-Spalten 1-6 werden parallel gespiegelt, falls dort noch keine Zeile</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17"/>
     <row r="18"/>
     <row r="19"/>
@@ -1968,9 +1377,9 @@
     <row r="49"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A12:J12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1982,143 +1391,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S199"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:S15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="97" min="1" max="1"/>
-    <col width="12" customWidth="1" style="97" min="2" max="2"/>
-    <col width="10" customWidth="1" style="97" min="3" max="3"/>
-    <col width="10" customWidth="1" style="97" min="4" max="4"/>
-    <col width="10" customWidth="1" style="97" min="5" max="5"/>
-    <col width="14" customWidth="1" style="97" min="6" max="6"/>
-    <col width="11" customWidth="1" style="97" min="7" max="7"/>
-    <col width="10" customWidth="1" style="97" min="8" max="8"/>
-    <col width="10" customWidth="1" style="97" min="9" max="9"/>
-    <col width="11" customWidth="1" style="97" min="10" max="10"/>
-    <col width="14" customWidth="1" style="97" min="11" max="11"/>
-    <col width="11" customWidth="1" style="97" min="12" max="12"/>
-    <col width="9" customWidth="1" style="97" min="13" max="13"/>
-    <col width="11" customWidth="1" style="97" min="14" max="14"/>
-    <col width="11" customWidth="1" style="97" min="15" max="15"/>
-    <col width="11" customWidth="1" style="97" min="16" max="16"/>
-    <col width="16" customWidth="1" style="97" min="17" max="17"/>
-    <col width="24" customWidth="1" style="97" min="18" max="18"/>
-    <col width="18" customWidth="1" style="97" min="19" max="19"/>
+    <col width="10" customWidth="1" style="44" min="1" max="1"/>
+    <col width="12" customWidth="1" style="44" min="2" max="2"/>
+    <col width="10" customWidth="1" style="44" min="3" max="5"/>
+    <col width="14" customWidth="1" style="44" min="6" max="6"/>
+    <col width="11" customWidth="1" style="44" min="7" max="7"/>
+    <col width="10" customWidth="1" style="44" min="8" max="9"/>
+    <col width="11" customWidth="1" style="44" min="10" max="10"/>
+    <col width="14" customWidth="1" style="44" min="11" max="11"/>
+    <col width="11" customWidth="1" style="44" min="12" max="12"/>
+    <col width="9" customWidth="1" style="44" min="13" max="13"/>
+    <col width="11" customWidth="1" style="44" min="14" max="16"/>
+    <col width="16" customWidth="1" style="44" min="17" max="17"/>
+    <col width="24" customWidth="1" style="44" min="18" max="18"/>
+    <col width="18" customWidth="1" style="44" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="136" t="inlineStr">
+    <row r="1" ht="19" customHeight="1" s="44">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>📊 Quartals-Bewertungen (Input + Output in einem Sheet)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="97">
-      <c r="A3" s="164" t="inlineStr">
+    <row r="3" ht="45" customHeight="1" s="44">
+      <c r="A3" s="57" t="inlineStr">
         <is>
           <t>Du trägst nur die GELBEN Spalten ein (Zufriedenheit + MediFox-IST). Der Rest wird beim Q-End-Lauf (8. Tag des Folge-Monats) automatisch vom Code befüllt. Status-Spalte zeigt was noch fehlt oder ob Diff &gt; 2 %.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="163" t="inlineStr">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>🟡 GELB = manuell von dir · 🟦 HELLBLAU = Code befüllt automatisch</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1" s="97">
-      <c r="A7" s="165" t="inlineStr">
+    <row r="7" ht="28" customHeight="1" s="44">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>Quartal</t>
         </is>
       </c>
-      <c r="B7" s="165" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="C7" s="165" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Rücken</t>
         </is>
       </c>
-      <c r="D7" s="165" t="inlineStr">
+      <c r="D7" s="37" t="inlineStr">
         <is>
           <t>Komm</t>
         </is>
       </c>
-      <c r="E7" s="165" t="inlineStr">
+      <c r="E7" s="37" t="inlineStr">
         <is>
           <t>eNPS</t>
         </is>
       </c>
-      <c r="F7" s="165" t="inlineStr">
+      <c r="F7" s="37" t="inlineStr">
         <is>
           <t>MediFox-IST €</t>
         </is>
       </c>
-      <c r="G7" s="165" t="inlineStr">
+      <c r="G7" s="37" t="inlineStr">
         <is>
           <t>Zufr-Score</t>
         </is>
       </c>
-      <c r="H7" s="165" t="inlineStr">
+      <c r="H7" s="37" t="inlineStr">
         <is>
           <t>Vstd ber</t>
         </is>
       </c>
-      <c r="I7" s="165" t="inlineStr">
+      <c r="I7" s="37" t="inlineStr">
         <is>
           <t>Abw ber</t>
         </is>
       </c>
-      <c r="J7" s="165" t="inlineStr">
+      <c r="J7" s="37" t="inlineStr">
         <is>
           <t>Feiertage h</t>
         </is>
       </c>
-      <c r="K7" s="165" t="inlineStr">
+      <c r="K7" s="37" t="inlineStr">
         <is>
           <t>IST €</t>
         </is>
       </c>
-      <c r="L7" s="165" t="inlineStr">
+      <c r="L7" s="37" t="inlineStr">
         <is>
           <t>verfueg h</t>
         </is>
       </c>
-      <c r="M7" s="165" t="inlineStr">
+      <c r="M7" s="37" t="inlineStr">
         <is>
           <t>€/h</t>
         </is>
       </c>
-      <c r="N7" s="165" t="inlineStr">
+      <c r="N7" s="37" t="inlineStr">
         <is>
           <t>Rechn-Stufe</t>
         </is>
       </c>
-      <c r="O7" s="165" t="inlineStr">
+      <c r="O7" s="37" t="inlineStr">
         <is>
           <t>Tats-Stufe</t>
         </is>
       </c>
-      <c r="P7" s="165" t="inlineStr">
+      <c r="P7" s="37" t="inlineStr">
         <is>
           <t>Probezeit</t>
         </is>
       </c>
-      <c r="Q7" s="165" t="inlineStr">
+      <c r="Q7" s="37" t="inlineStr">
         <is>
           <t>Diff € (NocoDB−MediFox)</t>
         </is>
       </c>
-      <c r="R7" s="165" t="inlineStr">
+      <c r="R7" s="37" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="S7" s="165" t="inlineStr">
+      <c r="S7" s="37" t="inlineStr">
         <is>
           <t>Berechnet am</t>
         </is>
@@ -2135,57 +1539,57 @@
           <t>Laura</t>
         </is>
       </c>
-      <c r="C8" s="144" t="n">
+      <c r="C8" s="51" t="n">
         <v>8.5</v>
       </c>
-      <c r="D8" s="144" t="n">
+      <c r="D8" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="144" t="n">
+      <c r="E8" s="51" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="F8" s="166" t="n">
+      <c r="F8" s="60" t="n">
         <v>299437</v>
       </c>
-      <c r="G8" s="167" t="n">
+      <c r="G8" s="39" t="n">
         <v>8.52</v>
       </c>
-      <c r="H8" s="167" t="n">
+      <c r="H8" s="39" t="n">
         <v>4686.3</v>
       </c>
-      <c r="I8" s="167" t="n">
+      <c r="I8" s="39" t="n">
         <v>554.8</v>
       </c>
-      <c r="J8" s="167" t="n"/>
-      <c r="K8" s="168" t="n">
+      <c r="J8" s="39" t="n"/>
+      <c r="K8" s="61" t="n">
         <v>291941</v>
       </c>
-      <c r="L8" s="167" t="n">
+      <c r="L8" s="39" t="n">
         <v>4131.5</v>
       </c>
-      <c r="M8" s="167" t="n">
+      <c r="M8" s="39" t="n">
         <v>70.66</v>
       </c>
-      <c r="N8" s="167" t="n">
+      <c r="N8" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="167" t="n">
+      <c r="O8" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="P8" s="167" t="inlineStr">
+      <c r="P8" s="39" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="Q8" s="168" t="n">
+      <c r="Q8" s="61" t="n">
         <v>-7496</v>
       </c>
-      <c r="R8" s="167" t="inlineStr">
+      <c r="R8" s="39" t="inlineStr">
         <is>
           <t>🔒 Q1 historisch eingefroren</t>
         </is>
       </c>
-      <c r="S8" s="167" t="inlineStr">
+      <c r="S8" s="39" t="inlineStr">
         <is>
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
@@ -2202,57 +1606,57 @@
           <t>Marleen</t>
         </is>
       </c>
-      <c r="C9" s="144" t="n">
+      <c r="C9" s="51" t="n">
         <v>8.5</v>
       </c>
-      <c r="D9" s="144" t="n">
+      <c r="D9" s="51" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="E9" s="144" t="n">
+      <c r="E9" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="166" t="n">
+      <c r="F9" s="60" t="n">
         <v>351752</v>
       </c>
-      <c r="G9" s="167" t="n">
+      <c r="G9" s="39" t="n">
         <v>8.24</v>
       </c>
-      <c r="H9" s="167" t="n">
+      <c r="H9" s="39" t="n">
         <v>5343.5</v>
       </c>
-      <c r="I9" s="167" t="n">
+      <c r="I9" s="39" t="n">
         <v>293.5</v>
       </c>
-      <c r="J9" s="167" t="n"/>
-      <c r="K9" s="168" t="n">
+      <c r="J9" s="39" t="n"/>
+      <c r="K9" s="61" t="n">
         <v>337924</v>
       </c>
-      <c r="L9" s="167" t="n">
+      <c r="L9" s="39" t="n">
         <v>5050</v>
       </c>
-      <c r="M9" s="167" t="n">
+      <c r="M9" s="39" t="n">
         <v>66.92</v>
       </c>
-      <c r="N9" s="167" t="n">
+      <c r="N9" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="O9" s="167" t="n">
+      <c r="O9" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="P9" s="167" t="inlineStr">
+      <c r="P9" s="39" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="Q9" s="168" t="n">
+      <c r="Q9" s="61" t="n">
         <v>-13828</v>
       </c>
-      <c r="R9" s="167" t="inlineStr">
+      <c r="R9" s="39" t="inlineStr">
         <is>
           <t>🔒 Q1 historisch eingefroren</t>
         </is>
       </c>
-      <c r="S9" s="167" t="inlineStr">
+      <c r="S9" s="39" t="inlineStr">
         <is>
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
@@ -2269,41 +1673,41 @@
           <t>Luise</t>
         </is>
       </c>
-      <c r="C10" s="144" t="n">
+      <c r="C10" s="51" t="n">
         <v>8.5</v>
       </c>
-      <c r="D10" s="144" t="n">
+      <c r="D10" s="51" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="E10" s="144" t="n"/>
-      <c r="F10" s="166" t="n">
+      <c r="E10" s="51" t="n"/>
+      <c r="F10" s="60" t="n">
         <v>351752</v>
       </c>
-      <c r="G10" s="167" t="n"/>
-      <c r="H10" s="167" t="n"/>
-      <c r="I10" s="167" t="n"/>
-      <c r="J10" s="167" t="n"/>
-      <c r="K10" s="168" t="n"/>
-      <c r="L10" s="167" t="n"/>
-      <c r="M10" s="167" t="n"/>
-      <c r="N10" s="167" t="n">
+      <c r="G10" s="39" t="n"/>
+      <c r="H10" s="39" t="n"/>
+      <c r="I10" s="39" t="n"/>
+      <c r="J10" s="39" t="n"/>
+      <c r="K10" s="61" t="n"/>
+      <c r="L10" s="39" t="n"/>
+      <c r="M10" s="39" t="n"/>
+      <c r="N10" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="O10" s="167" t="n">
+      <c r="O10" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="P10" s="167" t="inlineStr">
+      <c r="P10" s="39" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="Q10" s="168" t="n"/>
-      <c r="R10" s="167" t="inlineStr">
+      <c r="Q10" s="61" t="n"/>
+      <c r="R10" s="39" t="inlineStr">
         <is>
           <t>🔒 Q1 historisch eingefroren</t>
         </is>
       </c>
-      <c r="S10" s="167" t="inlineStr">
+      <c r="S10" s="39" t="inlineStr">
         <is>
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
@@ -2320,45 +1724,45 @@
           <t>Max</t>
         </is>
       </c>
-      <c r="C11" s="144" t="n">
+      <c r="C11" s="51" t="n">
         <v>8.5</v>
       </c>
-      <c r="D11" s="144" t="n">
+      <c r="D11" s="51" t="n">
         <v>7.8</v>
       </c>
-      <c r="E11" s="144" t="n">
+      <c r="E11" s="51" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="F11" s="166" t="n">
+      <c r="F11" s="60" t="n">
         <v>299437</v>
       </c>
-      <c r="G11" s="167" t="n">
+      <c r="G11" s="39" t="n">
         <v>8.539999999999999</v>
       </c>
-      <c r="H11" s="167" t="n"/>
-      <c r="I11" s="167" t="n"/>
-      <c r="J11" s="167" t="n"/>
-      <c r="K11" s="168" t="n"/>
-      <c r="L11" s="167" t="n"/>
-      <c r="M11" s="167" t="n"/>
-      <c r="N11" s="167" t="n">
+      <c r="H11" s="39" t="n"/>
+      <c r="I11" s="39" t="n"/>
+      <c r="J11" s="39" t="n"/>
+      <c r="K11" s="61" t="n"/>
+      <c r="L11" s="39" t="n"/>
+      <c r="M11" s="39" t="n"/>
+      <c r="N11" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="O11" s="167" t="n">
+      <c r="O11" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="P11" s="167" t="inlineStr">
+      <c r="P11" s="39" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="Q11" s="168" t="n"/>
-      <c r="R11" s="167" t="inlineStr">
+      <c r="Q11" s="61" t="n"/>
+      <c r="R11" s="39" t="inlineStr">
         <is>
           <t>🔒 Q1 historisch eingefroren</t>
         </is>
       </c>
-      <c r="S11" s="167" t="inlineStr">
+      <c r="S11" s="39" t="inlineStr">
         <is>
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
@@ -2375,11 +1779,11 @@
           <t>Laura</t>
         </is>
       </c>
-      <c r="C12" s="144" t="n"/>
-      <c r="D12" s="144" t="n"/>
-      <c r="E12" s="144" t="n"/>
-      <c r="F12" s="144" t="n"/>
-      <c r="R12" s="144" t="inlineStr">
+      <c r="C12" s="51" t="n"/>
+      <c r="D12" s="51" t="n"/>
+      <c r="E12" s="51" t="n"/>
+      <c r="F12" s="51" t="n"/>
+      <c r="R12" s="51" t="inlineStr">
         <is>
           <t>⏳ wartet auf Q-End-Lauf am 8.7.2026</t>
         </is>
@@ -2396,11 +1800,11 @@
           <t>Marleen</t>
         </is>
       </c>
-      <c r="C13" s="144" t="n"/>
-      <c r="D13" s="144" t="n"/>
-      <c r="E13" s="144" t="n"/>
-      <c r="F13" s="144" t="n"/>
-      <c r="R13" s="144" t="inlineStr">
+      <c r="C13" s="51" t="n"/>
+      <c r="D13" s="51" t="n"/>
+      <c r="E13" s="51" t="n"/>
+      <c r="F13" s="51" t="n"/>
+      <c r="R13" s="51" t="inlineStr">
         <is>
           <t>⏳ wartet auf Q-End-Lauf am 8.7.2026</t>
         </is>
@@ -2417,11 +1821,11 @@
           <t>Luise</t>
         </is>
       </c>
-      <c r="C14" s="144" t="n"/>
-      <c r="D14" s="144" t="n"/>
-      <c r="E14" s="144" t="n"/>
-      <c r="F14" s="144" t="n"/>
-      <c r="R14" s="144" t="inlineStr">
+      <c r="C14" s="51" t="n"/>
+      <c r="D14" s="51" t="n"/>
+      <c r="E14" s="51" t="n"/>
+      <c r="F14" s="51" t="n"/>
+      <c r="R14" s="51" t="inlineStr">
         <is>
           <t>⏳ wartet auf Q-End-Lauf am 8.7.2026</t>
         </is>
@@ -2438,400 +1842,16 @@
           <t>Max</t>
         </is>
       </c>
-      <c r="C15" s="144" t="n"/>
-      <c r="D15" s="144" t="n"/>
-      <c r="E15" s="144" t="n"/>
-      <c r="F15" s="144" t="n"/>
-      <c r="R15" s="144" t="inlineStr">
+      <c r="C15" s="51" t="n"/>
+      <c r="D15" s="51" t="n"/>
+      <c r="E15" s="51" t="n"/>
+      <c r="F15" s="51" t="n"/>
+      <c r="R15" s="51" t="inlineStr">
         <is>
           <t>⏳ wartet auf Q-End-Lauf am 8.7.2026</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-Q2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Laura</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>5198.4</v>
-      </c>
-      <c r="I16" t="n">
-        <v>721</v>
-      </c>
-      <c r="J16" t="n">
-        <v>343.5</v>
-      </c>
-      <c r="K16" t="n">
-        <v>265339</v>
-      </c>
-      <c r="L16" t="n">
-        <v>4133.9</v>
-      </c>
-      <c r="M16" t="n">
-        <v>64.19</v>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>⏳ Zufriedenheit fehlt</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>2026-07-08 05:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-Q2</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Marleen</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>7528.9</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1346.5</v>
-      </c>
-      <c r="J17" t="n">
-        <v>440.5</v>
-      </c>
-      <c r="K17" t="n">
-        <v>371864</v>
-      </c>
-      <c r="L17" t="n">
-        <v>5741.9</v>
-      </c>
-      <c r="M17" t="n">
-        <v>64.76000000000001</v>
-      </c>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>⏳ Zufriedenheit fehlt</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>2026-07-08 05:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-Q2</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Luise</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>7528.9</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1346.5</v>
-      </c>
-      <c r="J18" t="n">
-        <v>440.5</v>
-      </c>
-      <c r="K18" t="n">
-        <v>371864</v>
-      </c>
-      <c r="L18" t="n">
-        <v>5741.9</v>
-      </c>
-      <c r="M18" t="n">
-        <v>64.76000000000001</v>
-      </c>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>⏳ Zufriedenheit fehlt</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>2026-07-08 05:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-Q2</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>5198.4</v>
-      </c>
-      <c r="I19" t="n">
-        <v>721</v>
-      </c>
-      <c r="J19" t="n">
-        <v>343.5</v>
-      </c>
-      <c r="K19" t="n">
-        <v>265339</v>
-      </c>
-      <c r="L19" t="n">
-        <v>4133.9</v>
-      </c>
-      <c r="M19" t="n">
-        <v>64.19</v>
-      </c>
-      <c r="N19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>⏳ Zufriedenheit fehlt</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>2026-07-08 05:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2852,15 +1872,15 @@
   <dimension ref="B2:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="2" customWidth="1" style="97" min="1" max="1"/>
-    <col width="38" customWidth="1" style="97" min="2" max="2"/>
-    <col width="2" customWidth="1" style="97" min="3" max="3"/>
-    <col width="16" customWidth="1" style="97" min="4" max="4"/>
-    <col width="2" customWidth="1" style="97" min="5" max="5"/>
-    <col width="24" customWidth="1" style="97" min="6" max="6"/>
+    <col width="2" customWidth="1" style="44" min="1" max="1"/>
+    <col width="38" customWidth="1" style="44" min="2" max="2"/>
+    <col width="2" customWidth="1" style="44" min="3" max="3"/>
+    <col width="16" customWidth="1" style="44" min="4" max="4"/>
+    <col width="2" customWidth="1" style="44" min="5" max="5"/>
+    <col width="24" customWidth="1" style="44" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="2" ht="20" customHeight="1" s="97">
+    <row r="2" ht="20" customHeight="1" s="44">
       <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Parameter</t>
@@ -2935,7 +1955,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="48" t="n"/>
+      <c r="C9" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2953,10 +1973,10 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="8" customWidth="1" style="97" min="1" max="1"/>
-    <col width="16" customWidth="1" style="97" min="2" max="2"/>
-    <col width="14" customWidth="1" style="97" min="4" max="4"/>
-    <col width="12" customWidth="1" style="97" min="5" max="5"/>
+    <col width="8" customWidth="1" style="44" min="1" max="1"/>
+    <col width="16" customWidth="1" style="44" min="2" max="2"/>
+    <col width="14" customWidth="1" style="44" min="4" max="4"/>
+    <col width="12" customWidth="1" style="44" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2977,7 +1997,7 @@
           <t>Zulage %</t>
         </is>
       </c>
-      <c r="F1" s="59" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
         <is>
           <t>€/60min Therapie</t>
         </is>
@@ -2994,7 +2014,7 @@
       <c r="E2" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="131" t="n">
+      <c r="F2" s="62" t="n">
         <v>61.17</v>
       </c>
     </row>
@@ -3009,7 +2029,7 @@
       <c r="E3" s="8" t="n">
         <v>0.11</v>
       </c>
-      <c r="F3" s="131" t="n">
+      <c r="F3" s="62" t="n">
         <v>66.54000000000001</v>
       </c>
     </row>
@@ -3024,7 +2044,7 @@
       <c r="E4" s="8" t="n">
         <v>0.22</v>
       </c>
-      <c r="F4" s="131" t="n">
+      <c r="F4" s="62" t="n">
         <v>72.64</v>
       </c>
     </row>
@@ -3039,7 +2059,7 @@
       <c r="E5" s="8" t="n">
         <v>0.33</v>
       </c>
-      <c r="F5" s="131" t="n">
+      <c r="F5" s="62" t="n">
         <v>77.28</v>
       </c>
     </row>
@@ -3054,7 +2074,7 @@
       <c r="E6" s="8" t="n">
         <v>0.44</v>
       </c>
-      <c r="F6" s="131" t="n">
+      <c r="F6" s="62" t="n">
         <v>84.11</v>
       </c>
     </row>
@@ -3069,21 +2089,21 @@
       <c r="E7" s="8" t="n">
         <v>0.55</v>
       </c>
-      <c r="F7" s="131" t="n">
+      <c r="F7" s="62" t="n">
         <v>89.48</v>
       </c>
     </row>
     <row r="8"/>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="113" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
         <is>
           <t>Die €/60min-Spalte zeigt Umsatz pro Therapie-Stunde (Bundle-unabhängig, = IST ÷ verfügbare Zeit). Hinweis: Spalte „Leistungsindex" entfiel mit v18 — Stufen-Zuordnung läuft jetzt ausschließlich über €/60min.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="35" customHeight="1" s="97"/>
-    <row r="97" ht="51" customHeight="1" s="97"/>
+    <row r="11" ht="35" customHeight="1" s="44"/>
+    <row r="97" ht="51" customHeight="1" s="44"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A10:F10"/>
@@ -3103,9 +2123,9 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="6" customWidth="1" style="97" min="1" max="1"/>
-    <col width="14" customWidth="1" style="97" min="2" max="3"/>
-    <col width="16" customWidth="1" style="97" min="4" max="4"/>
+    <col width="6" customWidth="1" style="44" min="1" max="1"/>
+    <col width="14" customWidth="1" style="44" min="2" max="3"/>
+    <col width="16" customWidth="1" style="44" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3501,689 +2521,689 @@
   <dimension ref="B1:F99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="97" min="1" max="1"/>
-    <col width="28" customWidth="1" style="97" min="2" max="2"/>
-    <col width="34" customWidth="1" style="97" min="3" max="3"/>
-    <col width="28" customWidth="1" style="97" min="4" max="4"/>
-    <col width="14" customWidth="1" style="97" min="5" max="6"/>
+    <col width="2" customWidth="1" style="44" min="1" max="1"/>
+    <col width="28" customWidth="1" style="44" min="2" max="2"/>
+    <col width="34" customWidth="1" style="44" min="3" max="3"/>
+    <col width="28" customWidth="1" style="44" min="4" max="4"/>
+    <col width="14" customWidth="1" style="44" min="5" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" s="97">
-      <c r="B1" s="106" t="inlineStr">
+    <row r="1" ht="40" customHeight="1" s="44">
+      <c r="B1" s="50" t="inlineStr">
         <is>
           <t>Wie funktioniert dein Gehalt?</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" s="97">
-      <c r="B2" s="102" t="inlineStr">
+    <row r="2" ht="22" customHeight="1" s="44">
+      <c r="B2" s="46" t="inlineStr">
         <is>
           <t>Schritt für Schritt: vom Mindestgehalt bis zur variablen Zulage.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" s="97">
-      <c r="B4" s="100" t="inlineStr">
+    <row r="4" ht="28" customHeight="1" s="44">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>1. Dein Gehalt besteht aus drei Teilen</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" s="97">
-      <c r="B6" s="105" t="inlineStr">
+    <row r="6" ht="22" customHeight="1" s="44">
+      <c r="B6" s="49" t="inlineStr">
         <is>
           <t>A) Sockelgehalt</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" s="97">
-      <c r="B7" s="101" t="inlineStr">
+    <row r="7" ht="22" customHeight="1" s="44">
+      <c r="B7" s="45" t="inlineStr">
         <is>
           <t>40.000 € pro Jahr bei Vollzeit (40 h/Woche). Bei Teilzeit anteilig (26 h = 26/40 × 40.000 = 26.000 €).</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" s="97">
-      <c r="B9" s="105" t="inlineStr">
+    <row r="9" ht="22" customHeight="1" s="44">
+      <c r="B9" s="49" t="inlineStr">
         <is>
           <t>B) Bundle-Zulage (je nach Größe deines Teams)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" s="97">
-      <c r="B10" s="101" t="inlineStr">
+    <row r="10" ht="22" customHeight="1" s="44">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>Je mehr Therapeuten in deinem Bundle arbeiten, desto höher dein Gehalt.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="35" customHeight="1" s="97">
-      <c r="B11" s="101" t="inlineStr">
+    <row r="11" ht="35" customHeight="1" s="44">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>Wir rechnen nicht nach Anzahl Köpfen, sondern nach Stunden: die gesamten Wochenstunden aller TH im Bundle geteilt durch 30 — weil 30 h der übliche Vacura-Schnitt für einen TH ist. So ergibt sich dein »TH-Äquivalent«.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" s="97">
-      <c r="B12" s="102" t="inlineStr">
+    <row r="12" ht="22" customHeight="1" s="44">
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>Beispiel: 3 Therapeuten à 40 h + 2 à 30 h = 180 h ÷ 30 = 6 TH-Äquivalente.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" s="97">
-      <c r="B13" s="101" t="inlineStr">
+    <row r="13" ht="22" customHeight="1" s="44">
+      <c r="B13" s="45" t="inlineStr">
         <is>
           <t>Pro TH-Äquivalent bekommst du 250 € (für die ersten 4) bzw. 400 € (für 5–9) bzw. 700 € (ab 10) zusätzlich pro Jahr.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" s="97">
-      <c r="B15" s="105" t="inlineStr">
+    <row r="15" ht="22" customHeight="1" s="44">
+      <c r="B15" s="49" t="inlineStr">
         <is>
           <t>C) Variable Zulage</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1" s="97">
-      <c r="B16" s="101" t="inlineStr">
+    <row r="16" ht="22" customHeight="1" s="44">
+      <c r="B16" s="45" t="inlineStr">
         <is>
           <t>0 % bis 55 % Zulage auf dein Basis-Gehalt (= Sockel + Bundle-Zulage). Die 6 Stufen siehst du gleich in Abschnitt 2.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1" s="97">
-      <c r="B18" s="104" t="inlineStr">
+    <row r="18" ht="22" customHeight="1" s="44">
+      <c r="B18" s="48" t="inlineStr">
         <is>
           <t>Beispiel-Rechnung für eine Vollzeit-PM (40 h/Wo) mit 8 TH-Äquivalenten im Bundle:</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1" s="97">
-      <c r="B19" s="101" t="inlineStr">
+    <row r="19" ht="22" customHeight="1" s="44">
+      <c r="B19" s="45" t="inlineStr">
         <is>
           <t>• Sockel: 40.000 €</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1" s="97">
-      <c r="B20" s="101" t="inlineStr">
+    <row r="20" ht="22" customHeight="1" s="44">
+      <c r="B20" s="45" t="inlineStr">
         <is>
           <t>• Bundle-Zulage (8 TH-Äqui → kumuliert 2.600 €): + 2.600 €   →   Basis = 42.600 €</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1" s="97">
-      <c r="B21" s="105" t="inlineStr">
+    <row r="21" ht="22" customHeight="1" s="44">
+      <c r="B21" s="49" t="inlineStr">
         <is>
           <t>• Bei Stufe 3 (+22 % variable Zulage): 42.600 € × 1,22 = 51.972 € pro Jahr = 4.331 € pro Monat</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1" s="97">
-      <c r="B23" s="100" t="inlineStr">
+    <row r="23" ht="28" customHeight="1" s="44">
+      <c r="B23" s="43" t="inlineStr">
         <is>
           <t>2. Die 6 Stufen im Überblick</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1" s="97">
-      <c r="B25" s="102" t="inlineStr">
+    <row r="25" ht="22" customHeight="1" s="44">
+      <c r="B25" s="46" t="inlineStr">
         <is>
           <t>Jede Stufe entspricht einer festen variablen Zulage auf dein Basis-Gehalt:</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1" s="97">
-      <c r="B27" s="57" t="inlineStr">
+    <row r="27" ht="24" customHeight="1" s="44">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Stufe</t>
         </is>
       </c>
-      <c r="C27" s="57" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D27" s="57" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Zulage %</t>
         </is>
       </c>
-      <c r="E27" s="57" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Beispielgehalt Vollzeit, 8 TH</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1" s="97">
-      <c r="B28" s="61" t="inlineStr">
+    <row r="28" ht="24" customHeight="1" s="44">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C28" s="61" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="D28" s="61" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>0 %</t>
         </is>
       </c>
-      <c r="E28" s="62" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>42.600 €</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1" s="97">
-      <c r="B29" s="63" t="inlineStr">
+    <row r="29" ht="24" customHeight="1" s="44">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C29" s="63" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Gut</t>
         </is>
       </c>
-      <c r="D29" s="63" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>11 %</t>
         </is>
       </c>
-      <c r="E29" s="64" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>47.286 €</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1" s="97">
-      <c r="B30" s="61" t="inlineStr">
+    <row r="30" ht="24" customHeight="1" s="44">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C30" s="61" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Stark</t>
         </is>
       </c>
-      <c r="D30" s="61" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>22 %</t>
         </is>
       </c>
-      <c r="E30" s="62" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>51.972 €</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1" s="97">
-      <c r="B31" s="63" t="inlineStr">
+    <row r="31" ht="24" customHeight="1" s="44">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C31" s="63" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Sehr stark</t>
         </is>
       </c>
-      <c r="D31" s="63" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>33 %</t>
         </is>
       </c>
-      <c r="E31" s="64" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>56.658 €</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1" s="97">
-      <c r="B32" s="61" t="inlineStr">
+    <row r="32" ht="24" customHeight="1" s="44">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C32" s="61" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Exzellent</t>
         </is>
       </c>
-      <c r="D32" s="61" t="inlineStr">
+      <c r="D32" s="18" t="inlineStr">
         <is>
           <t>44 %</t>
         </is>
       </c>
-      <c r="E32" s="62" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>61.344 €</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1" s="97">
-      <c r="B33" s="65" t="inlineStr">
+    <row r="33" ht="24" customHeight="1" s="44">
+      <c r="B33" s="22" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C33" s="65" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>Herausragend</t>
         </is>
       </c>
-      <c r="D33" s="65" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>55 %</t>
         </is>
       </c>
-      <c r="E33" s="66" t="inlineStr">
+      <c r="E33" s="23" t="inlineStr">
         <is>
           <t>66.030 €</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1" s="97">
-      <c r="B36" s="100" t="inlineStr">
+    <row r="36" ht="28" customHeight="1" s="44">
+      <c r="B36" s="43" t="inlineStr">
         <is>
           <t>3. Wie ergibt sich deine Stufe?</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1" s="97">
-      <c r="B38" s="101" t="inlineStr">
+    <row r="38" ht="22" customHeight="1" s="44">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>Deine Stufe steht, wenn zwei Sachen gleichzeitig stimmen:</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1" s="97">
-      <c r="B40" s="105" t="inlineStr">
+    <row r="40" ht="22" customHeight="1" s="44">
+      <c r="B40" s="49" t="inlineStr">
         <is>
           <t>Bedingung 1 — Wirtschaftlich:</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1" s="97">
-      <c r="B41" s="101" t="inlineStr">
+    <row r="41" ht="22" customHeight="1" s="44">
+      <c r="B41" s="45" t="inlineStr">
         <is>
           <t>Dein Bundle muss einen bestimmten Umsatz pro Therapie-Stunde erwirtschaften.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1" s="97">
-      <c r="B42" s="101" t="inlineStr">
+    <row r="42" ht="22" customHeight="1" s="44">
+      <c r="B42" s="45" t="inlineStr">
         <is>
           <t>Zum Beispiel: Für Stufe 3 brauchst du ca. 73 €/Stunde, für Stufe 5 ca. 84 €/Stunde. Details dazu in Abschnitt 4.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1" s="97">
-      <c r="B44" s="105" t="inlineStr">
+    <row r="44" ht="22" customHeight="1" s="44">
+      <c r="B44" s="49" t="inlineStr">
         <is>
           <t>Bedingung 2 — Teamzufriedenheit:</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1" s="97">
-      <c r="B45" s="101" t="inlineStr">
+    <row r="45" ht="22" customHeight="1" s="44">
+      <c r="B45" s="45" t="inlineStr">
         <is>
           <t>Dein Team muss in der anonymen Quartals-Umfrage einen bestimmten Zufriedenheits-Score erreichen (Skala 0–10).</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1" s="97">
-      <c r="B46" s="101" t="inlineStr">
+    <row r="46" ht="22" customHeight="1" s="44">
+      <c r="B46" s="45" t="inlineStr">
         <is>
           <t>Zum Beispiel: Stufe 3 braucht ≥ 7,0 — Stufe 5 braucht ≥ 8,5.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1" s="97">
-      <c r="B48" s="103" t="inlineStr">
+    <row r="48" ht="22" customHeight="1" s="44">
+      <c r="B48" s="47" t="inlineStr">
         <is>
           <t>Beide Schwellen müssen erfüllt sein — nur wirtschaftlich stark ODER nur glückliches Team reicht nicht.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="22" customHeight="1" s="97">
-      <c r="B50" s="105" t="inlineStr">
+    <row r="50" ht="22" customHeight="1" s="44">
+      <c r="B50" s="49" t="inlineStr">
         <is>
           <t>Die Schwellen pro Stufe:</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="22" customHeight="1" s="97">
-      <c r="B52" s="57" t="inlineStr">
+    <row r="52" ht="22" customHeight="1" s="44">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>Stufe</t>
         </is>
       </c>
-      <c r="C52" s="57" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr">
         <is>
           <t>€/60min Therapie (min.)</t>
         </is>
       </c>
-      <c r="D52" s="57" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>Zufriedenheits-Score (min.)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1" s="97">
-      <c r="B53" s="63" t="inlineStr">
+    <row r="53" ht="22" customHeight="1" s="44">
+      <c r="B53" s="20" t="inlineStr">
         <is>
           <t>1 Basis</t>
         </is>
       </c>
-      <c r="C53" s="63" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
         <is>
           <t>61,17 €</t>
         </is>
       </c>
-      <c r="D53" s="63" t="inlineStr">
+      <c r="D53" s="20" t="inlineStr">
         <is>
           <t>5,0</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="22" customHeight="1" s="97">
-      <c r="B54" s="61" t="inlineStr">
+    <row r="54" ht="22" customHeight="1" s="44">
+      <c r="B54" s="18" t="inlineStr">
         <is>
           <t>2 Gut</t>
         </is>
       </c>
-      <c r="C54" s="61" t="inlineStr">
+      <c r="C54" s="18" t="inlineStr">
         <is>
           <t>66,54 €</t>
         </is>
       </c>
-      <c r="D54" s="61" t="inlineStr">
+      <c r="D54" s="18" t="inlineStr">
         <is>
           <t>6,0</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="22" customHeight="1" s="97">
-      <c r="B55" s="63" t="inlineStr">
+    <row r="55" ht="22" customHeight="1" s="44">
+      <c r="B55" s="20" t="inlineStr">
         <is>
           <t>3 Stark</t>
         </is>
       </c>
-      <c r="C55" s="63" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
         <is>
           <t>72,64 €</t>
         </is>
       </c>
-      <c r="D55" s="63" t="inlineStr">
+      <c r="D55" s="20" t="inlineStr">
         <is>
           <t>7,0</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1" s="97">
-      <c r="B56" s="61" t="inlineStr">
+    <row r="56" ht="22" customHeight="1" s="44">
+      <c r="B56" s="18" t="inlineStr">
         <is>
           <t>4 Sehr stark</t>
         </is>
       </c>
-      <c r="C56" s="61" t="inlineStr">
+      <c r="C56" s="18" t="inlineStr">
         <is>
           <t>77,28 €</t>
         </is>
       </c>
-      <c r="D56" s="61" t="inlineStr">
+      <c r="D56" s="18" t="inlineStr">
         <is>
           <t>8,0</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="22" customHeight="1" s="97">
-      <c r="B57" s="63" t="inlineStr">
+    <row r="57" ht="22" customHeight="1" s="44">
+      <c r="B57" s="20" t="inlineStr">
         <is>
           <t>5 Exzellent</t>
         </is>
       </c>
-      <c r="C57" s="63" t="inlineStr">
+      <c r="C57" s="20" t="inlineStr">
         <is>
           <t>84,11 €</t>
         </is>
       </c>
-      <c r="D57" s="63" t="inlineStr">
+      <c r="D57" s="20" t="inlineStr">
         <is>
           <t>8,5</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1" s="97">
-      <c r="B58" s="61" t="inlineStr">
+    <row r="58" ht="22" customHeight="1" s="44">
+      <c r="B58" s="18" t="inlineStr">
         <is>
           <t>6 Herausragend</t>
         </is>
       </c>
-      <c r="C58" s="61" t="inlineStr">
+      <c r="C58" s="18" t="inlineStr">
         <is>
           <t>89,48 €</t>
         </is>
       </c>
-      <c r="D58" s="61" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>8,5</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="28" customHeight="1" s="97">
-      <c r="B61" s="100" t="inlineStr">
+    <row r="61" ht="28" customHeight="1" s="44">
+      <c r="B61" s="43" t="inlineStr">
         <is>
           <t>4. Was bedeutet »€/60min Therapie«?</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="22" customHeight="1" s="97">
-      <c r="B63" s="101" t="inlineStr">
+    <row r="63" ht="22" customHeight="1" s="44">
+      <c r="B63" s="45" t="inlineStr">
         <is>
           <t>Das ist der Wert, an dem deine Leistung gemessen wird.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="22" customHeight="1" s="97">
-      <c r="B64" s="101" t="inlineStr">
+    <row r="64" ht="22" customHeight="1" s="44">
+      <c r="B64" s="45" t="inlineStr">
         <is>
           <t>Er sagt: Wie viel Umsatz macht dein Bundle durchschnittlich pro Stunde, in der ein TH tatsächlich arbeitet (also nicht im Urlaub oder in Fortbildung ist).</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="22" customHeight="1" s="97">
-      <c r="B66" s="103" t="inlineStr">
+    <row r="66" ht="22" customHeight="1" s="44">
+      <c r="B66" s="47" t="inlineStr">
         <is>
           <t>In einfachen Worten:</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="22" customHeight="1" s="97">
-      <c r="B67" s="103" t="inlineStr">
+    <row r="67" ht="22" customHeight="1" s="44">
+      <c r="B67" s="47" t="inlineStr">
         <is>
           <t>Gesamt-Umsatz deines Bundles im Quartal  ÷  alle verfügbaren Arbeitsstunden = €/60min</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="22" customHeight="1" s="97">
-      <c r="B69" s="101" t="inlineStr">
+    <row r="69" ht="22" customHeight="1" s="44">
+      <c r="B69" s="45" t="inlineStr">
         <is>
           <t>Verfügbare Arbeitsstunden = alle Vertragsstunden MINUS Urlaub, Fortbildung, Sonderurlaub.</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="22" customHeight="1" s="97">
-      <c r="B70" s="101" t="inlineStr">
+    <row r="70" ht="22" customHeight="1" s="44">
+      <c r="B70" s="45" t="inlineStr">
         <is>
           <t>Krankheit wird NICHT abgezogen — die ist schon als 10 %-Puffer im Modell einkalkuliert.</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="22" customHeight="1" s="97">
-      <c r="B72" s="102" t="inlineStr">
+    <row r="72" ht="22" customHeight="1" s="44">
+      <c r="B72" s="46" t="inlineStr">
         <is>
           <t>Zum Einordnen: Ein 60-min-GKV-Termin bringt ca. 95 €. Weil zwischen Terminen Zeit für Doku/Pausen bezahlt ist, liegt der Schnitt darunter.</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="28" customHeight="1" s="97">
-      <c r="B75" s="100" t="inlineStr">
+    <row r="75" ht="28" customHeight="1" s="44">
+      <c r="B75" s="43" t="inlineStr">
         <is>
           <t>5. Wie kommst du zur nächsten Stufe?</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="22" customHeight="1" s="97">
-      <c r="B77" s="101" t="inlineStr">
+    <row r="77" ht="22" customHeight="1" s="44">
+      <c r="B77" s="45" t="inlineStr">
         <is>
           <t>Drei Hebel, um den €/60min nach oben zu bekommen:</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="22" customHeight="1" s="97">
-      <c r="B78" s="102" t="inlineStr">
+    <row r="78" ht="22" customHeight="1" s="44">
+      <c r="B78" s="46" t="inlineStr">
         <is>
           <t>Hinweis: die Effekte sind Orientierungswerte (grobe Rechnung), keine exakt vorhergesagten Zahlen.</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="34" customHeight="1" s="97">
-      <c r="B80" s="57" t="inlineStr">
+    <row r="80" ht="34" customHeight="1" s="44">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>Hebel</t>
         </is>
       </c>
-      <c r="C80" s="57" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>Was machst du konkret?</t>
         </is>
       </c>
-      <c r="D80" s="57" t="inlineStr">
+      <c r="D80" s="15" t="inlineStr">
         <is>
           <t>Grober Effekt</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="34" customHeight="1" s="97">
-      <c r="B81" s="67" t="inlineStr">
+    <row r="81" ht="34" customHeight="1" s="44">
+      <c r="B81" s="24" t="inlineStr">
         <is>
           <t>Mehr Termine pro Woche</t>
         </is>
       </c>
-      <c r="C81" s="67" t="inlineStr">
+      <c r="C81" s="24" t="inlineStr">
         <is>
           <t>Auslastung erhöhen, neue Patienten gewinnen, Slots besser nutzen</t>
         </is>
       </c>
-      <c r="D81" s="67" t="inlineStr">
+      <c r="D81" s="24" t="inlineStr">
         <is>
           <t>+10 Termine/Wo → ca. +3 % Umsatz</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="34" customHeight="1" s="97">
-      <c r="B82" s="68" t="inlineStr">
+    <row r="82" ht="34" customHeight="1" s="44">
+      <c r="B82" s="25" t="inlineStr">
         <is>
           <t>Höherer PKV-Anteil</t>
         </is>
       </c>
-      <c r="C82" s="68" t="inlineStr">
+      <c r="C82" s="25" t="inlineStr">
         <is>
           <t>Privatpatienten aktiv ansprechen (PKV zahlt 1,7× den GKV-Tarif)</t>
         </is>
       </c>
-      <c r="D82" s="68" t="inlineStr">
+      <c r="D82" s="25" t="inlineStr">
         <is>
           <t>+1 %-Pkt PKV → ca. +0,7 % Umsatz</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="34" customHeight="1" s="97">
-      <c r="B83" s="67" t="inlineStr">
+    <row r="83" ht="34" customHeight="1" s="44">
+      <c r="B83" s="24" t="inlineStr">
         <is>
           <t>Krankenstand senken</t>
         </is>
       </c>
-      <c r="C83" s="67" t="inlineStr">
+      <c r="C83" s="24" t="inlineStr">
         <is>
           <t>Team-Gesundheit, gute Urlaubsplanung, keine Ansteckungsketten</t>
         </is>
       </c>
-      <c r="D83" s="67" t="inlineStr">
+      <c r="D83" s="24" t="inlineStr">
         <is>
           <t>−1 %-Pkt Krank → ca. +0,5 % Umsatz</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="22" customHeight="1" s="97">
-      <c r="B85" s="102" t="inlineStr">
+    <row r="85" ht="22" customHeight="1" s="44">
+      <c r="B85" s="46" t="inlineStr">
         <is>
           <t>Plus: Team-Zufriedenheits-Score hoch halten — ohne den bringt dir der beste Leistungsindex nichts.</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="28" customHeight="1" s="97">
-      <c r="B87" s="100" t="inlineStr">
+    <row r="87" ht="28" customHeight="1" s="44">
+      <c r="B87" s="43" t="inlineStr">
         <is>
           <t>6. Spezial-Regeln</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="22" customHeight="1" s="97">
-      <c r="B89" s="105" t="inlineStr">
+    <row r="89" ht="22" customHeight="1" s="44">
+      <c r="B89" s="49" t="inlineStr">
         <is>
           <t>Probezeit (erste 6 Monate):</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="22" customHeight="1" s="97">
-      <c r="B90" s="101" t="inlineStr">
+    <row r="90" ht="22" customHeight="1" s="44">
+      <c r="B90" s="45" t="inlineStr">
         <is>
           <t>Stufe ist fix auf 1 (Basis), Bundle-Zulage zählt nicht, Gehalt = Mindestgehalt. Nach 180 Tagen greift das Stufensystem.</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="22" customHeight="1" s="97">
-      <c r="B92" s="105" t="inlineStr">
+    <row r="92" ht="22" customHeight="1" s="44">
+      <c r="B92" s="49" t="inlineStr">
         <is>
           <t>Max ±1 Stufenwechsel pro Quartal:</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="22" customHeight="1" s="97">
-      <c r="B93" s="101" t="inlineStr">
+    <row r="93" ht="22" customHeight="1" s="44">
+      <c r="B93" s="45" t="inlineStr">
         <is>
           <t>Auch bei perfekter Performance kannst du pro Quartal nur eine Stufe steigen. Ein Abstieg ist auf −1 Stufe begrenzt.</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="22" customHeight="1" s="97">
-      <c r="B95" s="105" t="inlineStr">
+    <row r="95" ht="22" customHeight="1" s="44">
+      <c r="B95" s="49" t="inlineStr">
         <is>
           <t>Neuanfänger (neue TH im Bundle):</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="22" customHeight="1" s="97">
-      <c r="B96" s="101" t="inlineStr">
+    <row r="96" ht="22" customHeight="1" s="44">
+      <c r="B96" s="45" t="inlineStr">
         <is>
           <t>Frisch eingestellte TH zählen erst ab dem 29. Tag ihres Arbeitsverhältnisses — damit ihre Einarbeitung deinen €/60min-Wert nicht drückt.</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="51" customHeight="1" s="97"/>
-    <row r="98" ht="22" customHeight="1" s="97">
-      <c r="B98" s="105" t="n"/>
-    </row>
-    <row r="99" ht="22" customHeight="1" s="97">
-      <c r="B99" s="101" t="n"/>
+    <row r="97" ht="51" customHeight="1" s="44"/>
+    <row r="98" ht="22" customHeight="1" s="44">
+      <c r="B98" s="49" t="n"/>
+    </row>
+    <row r="99" ht="22" customHeight="1" s="44">
+      <c r="B99" s="45" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="49">
@@ -4191,9 +3211,9 @@
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B90:F90"/>
     <mergeCell ref="B72:F72"/>
-    <mergeCell ref="B90:F90"/>
-    <mergeCell ref="B25:F25"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B93:F93"/>

</xml_diff>

<commit_message>
Q2-Abschluss: ZI-Bepreisung (Valentin-Systematik) + Q2-Bewertung live
- termin_umsatz: (Dauer/15 + 1 VNB-ZI) × 18,98; thermisch 8,51; PKV ×2,0, SZ ×1,7;
  +4,11 % ab 01.07.2026; VO-Blattgebühr 10 € + Blanko-Pauschale 98,59 € in compute_quartal
  (Backtest vs. MediFox Q1+Q2: −4,4 bis +1,7 %)
- Q-End-Routine: Zufr-Score + Vorquartals-Stufe werden jetzt an compute_quartal
  durchgereicht (Bug: zufr fiel auf 0 → alle Stufe 1)
- compute_pm: verfueg aus Routine-Spalte 12 bzw. inkl. Feiertage-Spalte
- Dashboards dynamisch auf letztes abgeschlossenes Quartal (Q2 2026), Emily live
- Q2 2026 eingefroren; Ergebnis: Laura/Marleen Stufe 2, Probezeit-PMs Stufe 1

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4600" yWindow="-19780" windowWidth="24200" windowHeight="15120" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4600" yWindow="-19780" windowWidth="24200" windowHeight="15120" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Modell" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung Q-Wechsel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Stammdaten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quartals-Bewertungen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stufentabelle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-Zulagen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modell" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1786,13 +1786,13 @@
         <v>8.4</v>
       </c>
       <c r="F12" s="38" t="n">
-        <v>294446</v>
+        <v>287559</v>
       </c>
       <c r="G12" t="n">
         <v>8.48</v>
       </c>
       <c r="H12" t="n">
-        <v>5265.3</v>
+        <v>5228.9</v>
       </c>
       <c r="I12" t="n">
         <v>721</v>
@@ -1801,19 +1801,19 @@
         <v>343.5</v>
       </c>
       <c r="K12" t="n">
-        <v>266847</v>
+        <v>287559</v>
       </c>
       <c r="L12" t="n">
-        <v>4200.8</v>
+        <v>4164.4</v>
       </c>
       <c r="M12" t="n">
-        <v>63.52</v>
+        <v>69.05</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1821,16 +1821,16 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>-27599</v>
+        <v>0</v>
       </c>
       <c r="R12" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff -9.4 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-07-21 15:01</t>
+          <t>2026-07-22 10:18</t>
         </is>
       </c>
     </row>
@@ -1855,13 +1855,13 @@
         <v>7.8</v>
       </c>
       <c r="F13" s="38" t="n">
-        <v>424403</v>
+        <v>397312</v>
       </c>
       <c r="G13" t="n">
         <v>7.8</v>
       </c>
       <c r="H13" t="n">
-        <v>7478.6</v>
+        <v>7377.3</v>
       </c>
       <c r="I13" t="n">
         <v>1345.5</v>
@@ -1870,19 +1870,19 @@
         <v>440.5</v>
       </c>
       <c r="K13" t="n">
-        <v>373518</v>
+        <v>397312</v>
       </c>
       <c r="L13" t="n">
-        <v>5692.6</v>
+        <v>5591.3</v>
       </c>
       <c r="M13" t="n">
-        <v>65.61</v>
+        <v>71.06</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -1890,16 +1890,16 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>-50885</v>
+        <v>0</v>
       </c>
       <c r="R13" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff -12.0 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-07-21 15:01</t>
+          <t>2026-07-22 10:18</t>
         </is>
       </c>
     </row>
@@ -1924,13 +1924,13 @@
         <v>9.199999999999999</v>
       </c>
       <c r="F14" s="38" t="n">
-        <v>424403</v>
+        <v>397312</v>
       </c>
       <c r="G14" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>7478.6</v>
+        <v>7377.3</v>
       </c>
       <c r="I14" t="n">
         <v>1345.5</v>
@@ -1939,16 +1939,16 @@
         <v>440.5</v>
       </c>
       <c r="K14" t="n">
-        <v>373518</v>
+        <v>397312</v>
       </c>
       <c r="L14" t="n">
-        <v>5692.6</v>
+        <v>5591.3</v>
       </c>
       <c r="M14" t="n">
-        <v>65.61</v>
+        <v>71.06</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" t="n">
         <v>1</v>
@@ -1959,16 +1959,16 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>-50885</v>
+        <v>0</v>
       </c>
       <c r="R14" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff -12.0 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-07-21 15:01</t>
+          <t>2026-07-22 10:18</t>
         </is>
       </c>
     </row>
@@ -1993,13 +1993,13 @@
         <v>8.9</v>
       </c>
       <c r="F15" s="38" t="n">
-        <v>294446</v>
+        <v>287559</v>
       </c>
       <c r="G15" t="n">
         <v>9.08</v>
       </c>
       <c r="H15" t="n">
-        <v>5265.3</v>
+        <v>5228.9</v>
       </c>
       <c r="I15" t="n">
         <v>721</v>
@@ -2008,16 +2008,16 @@
         <v>343.5</v>
       </c>
       <c r="K15" t="n">
-        <v>266847</v>
+        <v>287559</v>
       </c>
       <c r="L15" t="n">
-        <v>4200.8</v>
+        <v>4164.4</v>
       </c>
       <c r="M15" t="n">
-        <v>63.52</v>
+        <v>69.05</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>
@@ -2028,16 +2028,16 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>-27599</v>
+        <v>0</v>
       </c>
       <c r="R15" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff -9.4 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-07-21 15:01</t>
+          <t>2026-07-22 10:18</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7478.6</v>
+        <v>7377.3</v>
       </c>
       <c r="I16" t="n">
         <v>1345.5</v>
@@ -2062,13 +2062,13 @@
         <v>440.5</v>
       </c>
       <c r="K16" t="n">
-        <v>373518</v>
+        <v>397312</v>
       </c>
       <c r="L16" t="n">
-        <v>5692.6</v>
+        <v>5591.3</v>
       </c>
       <c r="M16" t="n">
-        <v>65.61</v>
+        <v>71.06</v>
       </c>
       <c r="N16" t="n">
         <v>1</v>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-07-21 15:01</t>
+          <t>2026-07-22 10:18</t>
         </is>
       </c>
     </row>
@@ -3634,9 +3634,9 @@
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B90:F90"/>
     <mergeCell ref="B72:F72"/>
-    <mergeCell ref="B90:F90"/>
-    <mergeCell ref="B25:F25"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B93:F93"/>

</xml_diff>

<commit_message>
PM-Std-Bundle Laura/Max 65→70 + Probezeit-Hinweis im Dashboard + Bundle-Änderungs-Anleitung
- Stammdaten: Anteile Laura 40/70, Max 30/70 (vorher 108 % Überallokation bei 65)
- Dashboards: Probezeit-PMs sehen jetzt Hero-Badge + Erklärung im Einordnung-Block
  (Stufe fest auf 1 trotz erreichter Schwellen — war unerklärt verwirrend)
- ANLEITUNG: neuer Abschnitt 'Neuer Standort / Bundle-Änderung' (Excel + n8n-BUNDLES)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="2"/>
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="47" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D6" s="47" t="n">
         <v>45000</v>
@@ -1227,7 +1227,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="47" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D9" s="47" t="n">
         <v>40000</v>
@@ -1303,7 +1303,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
@@ -1339,39 +1338,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
@@ -1388,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S199"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="1"/>
@@ -2092,189 +2058,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2393,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="45" min="1" max="1"/>
@@ -2516,8 +2299,6 @@
         <v>89.48</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Q2-Tabelle auf finale Logik aktualisiert (gehaltsneutral) + wieder eingefroren
Q2-Zeilen neu gerechnet mit finalem Stand (ZI-Form, gelöschte erbrachte,
0,8×geplante Juni, VO-Pauschalen): Laura 69,89 €/h, Marleen 72,46 — Stufen
unverändert (2/2, Probezeit-Fälle 1), Status überall ✓ OK. Freeze wiederhergestellt.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -21,14 +21,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0\ \€"/>
+    <numFmt numFmtId="169" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -212,6 +213,12 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF666666"/>
+      <sz val="16"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -330,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -421,17 +428,17 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -455,6 +462,10 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -725,14 +736,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" s="45">
-      <c r="A1" s="44" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>📋 Anleitung Quartalswechsel — Was tun, wenn ein Quartal endet?</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" s="45">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>Diese Anleitung beschreibt die manuellen Schritte, die nach jedem Quartals-Ende notwendig sind, damit die PM-Bewertung für das Folge-Quartal greift.</t>
         </is>
@@ -1013,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="2"/>
@@ -1027,14 +1038,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" s="45">
-      <c r="A1" s="44" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>👥 PM-Stammdaten (Quelle der Wahrheit für PM-Liste)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1" s="45">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>Quelle der Wahrheit für die PM-Liste. Code liest beim Start automatisch.
 ➜ Neuen PM anlegen: einfach neue Zeile anhängen. Spalte 8 (Farbe), 9 (Token) und 10 (Aktiv) dürfen leer bleiben — werden beim nächsten Dashboard-Lauf automatisch befüllt. Token wird automatisch erzeugt und ins Excel zurückgeschrieben.</t>
@@ -1094,215 +1105,216 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" s="45">
-      <c r="A6" s="47" t="inlineStr">
+      <c r="A6" s="51" t="inlineStr">
         <is>
           <t>Laura</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="51" t="n">
         <v>40</v>
       </c>
-      <c r="C6" s="47" t="n">
+      <c r="C6" s="51" t="n">
         <v>70</v>
       </c>
-      <c r="D6" s="47" t="n">
+      <c r="D6" s="51" t="n">
         <v>45000</v>
       </c>
-      <c r="E6" s="47" t="n"/>
-      <c r="F6" s="47" t="inlineStr">
+      <c r="E6" s="51" t="n"/>
+      <c r="F6" s="51" t="inlineStr">
         <is>
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="G6" s="47" t="inlineStr">
+      <c r="G6" s="51" t="inlineStr">
         <is>
           <t>Laura, Max</t>
         </is>
       </c>
-      <c r="H6" s="47" t="inlineStr">
+      <c r="H6" s="51" t="inlineStr">
         <is>
           <t>#4CAF50</t>
         </is>
       </c>
-      <c r="I6" s="47" t="inlineStr">
+      <c r="I6" s="51" t="inlineStr">
         <is>
           <t>8278b207ba9e80605ae5f1604d696759</t>
         </is>
       </c>
-      <c r="J6" s="47" t="b">
+      <c r="J6" s="51" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" s="45">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>Marleen</t>
         </is>
       </c>
-      <c r="B7" s="47" t="n">
+      <c r="B7" s="51" t="n">
         <v>40</v>
       </c>
-      <c r="C7" s="47" t="n">
+      <c r="C7" s="51" t="n">
         <v>120</v>
       </c>
-      <c r="D7" s="47" t="n">
+      <c r="D7" s="51" t="n">
         <v>45000</v>
       </c>
-      <c r="E7" s="47" t="n"/>
-      <c r="F7" s="47" t="inlineStr">
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="inlineStr">
         <is>
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="G7" s="47" t="inlineStr">
+      <c r="G7" s="51" t="inlineStr">
         <is>
           <t>Marleen, Luise, Emily</t>
         </is>
       </c>
-      <c r="H7" s="47" t="inlineStr">
+      <c r="H7" s="51" t="inlineStr">
         <is>
           <t>#2196F3</t>
         </is>
       </c>
-      <c r="I7" s="47" t="inlineStr">
+      <c r="I7" s="51" t="inlineStr">
         <is>
           <t>0093979f8cf4df0f67ec20b6e35e6beb</t>
         </is>
       </c>
-      <c r="J7" s="47" t="b">
+      <c r="J7" s="51" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" s="45">
-      <c r="A8" s="47" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>Luise</t>
         </is>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="51" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="47" t="n">
+      <c r="C8" s="51" t="n">
         <v>120</v>
       </c>
-      <c r="D8" s="47" t="n">
+      <c r="D8" s="51" t="n">
         <v>40000</v>
       </c>
-      <c r="E8" s="47" t="inlineStr">
+      <c r="E8" s="51" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="F8" s="47" t="inlineStr">
+      <c r="F8" s="51" t="inlineStr">
         <is>
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="G8" s="47" t="inlineStr">
+      <c r="G8" s="51" t="inlineStr">
         <is>
           <t>Marleen, Luise, Emily</t>
         </is>
       </c>
-      <c r="H8" s="47" t="inlineStr">
+      <c r="H8" s="51" t="inlineStr">
         <is>
           <t>#9C27B0</t>
         </is>
       </c>
-      <c r="I8" s="47" t="inlineStr">
+      <c r="I8" s="51" t="inlineStr">
         <is>
           <t>52981192518b734a346928ed713bc015</t>
         </is>
       </c>
-      <c r="J8" s="47" t="b">
+      <c r="J8" s="51" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" s="45">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="B9" s="47" t="n">
+      <c r="B9" s="51" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="47" t="n">
+      <c r="C9" s="51" t="n">
         <v>70</v>
       </c>
-      <c r="D9" s="47" t="n">
+      <c r="D9" s="51" t="n">
         <v>40000</v>
       </c>
-      <c r="E9" s="47" t="inlineStr">
+      <c r="E9" s="51" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="F9" s="47" t="inlineStr">
+      <c r="F9" s="51" t="inlineStr">
         <is>
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="G9" s="47" t="inlineStr">
+      <c r="G9" s="51" t="inlineStr">
         <is>
           <t>Laura, Max</t>
         </is>
       </c>
-      <c r="H9" s="47" t="inlineStr">
+      <c r="H9" s="51" t="inlineStr">
         <is>
           <t>#FF9800</t>
         </is>
       </c>
-      <c r="I9" s="47" t="inlineStr">
+      <c r="I9" s="51" t="inlineStr">
         <is>
           <t>5051837ce5b8f243f109306f60136f17</t>
         </is>
       </c>
-      <c r="J9" s="47" t="b">
+      <c r="J9" s="51" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" s="45">
-      <c r="A10" s="47" t="inlineStr">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t>Emily</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="51" t="n">
         <v>40</v>
       </c>
-      <c r="C10" s="47" t="n">
+      <c r="C10" s="51" t="n">
         <v>120</v>
       </c>
-      <c r="D10" s="47" t="n">
+      <c r="D10" s="51" t="n">
         <v>40000</v>
       </c>
       <c r="E10" s="43" t="n">
         <v>46204</v>
       </c>
-      <c r="F10" s="47" t="inlineStr">
+      <c r="F10" s="51" t="inlineStr">
         <is>
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="G10" s="47" t="inlineStr">
+      <c r="G10" s="51" t="inlineStr">
         <is>
           <t>Marleen, Luise, Emily</t>
         </is>
       </c>
-      <c r="H10" s="47" t="inlineStr">
+      <c r="H10" s="51" t="inlineStr">
         <is>
           <t>#0D595A</t>
         </is>
       </c>
-      <c r="I10" s="47" t="inlineStr">
+      <c r="I10" s="51" t="inlineStr">
         <is>
           <t>34ff01c507e5f18ac55f03759f68f856</t>
         </is>
       </c>
-      <c r="J10" s="47" t="b">
+      <c r="J10" s="51" t="b">
         <v>1</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
@@ -1311,33 +1323,66 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>• Spalte 8 leer → Default-Farbe #0D595A (Vacura-Teal)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="46" t="inlineStr">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>• Spalte 9 leer → Token wird per secrets.token_hex(16) erzeugt + hier eingetragen</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>• Spalte 10 leer → Aktiv=Ja angenommen. Auf FALSE setzen um PM zu deaktivieren (z.B. Austritt)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="46" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>• Plus: Daten-Tab Stammdaten-Spalten 1-6 werden parallel gespiegelt, falls dort noch keine Zeile</t>
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
@@ -1354,7 +1399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S199"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="1"/>
@@ -1374,21 +1419,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" s="45">
-      <c r="A1" s="44" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>📊 Quartals-Bewertungen (Input + Output in einem Sheet)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" s="45">
-      <c r="A3" s="51" t="inlineStr">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>Du trägst nur die GELBEN Spalten ein (Zufriedenheit + MediFox-IST). Der Rest wird beim Q-End-Lauf (8. Tag des Folge-Monats) automatisch vom Code befüllt. Status-Spalte zeigt was noch fehlt oder ob Diff &gt; 2 %.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>🟡 GELB = manuell von dir · 🟦 HELLBLAU = Code befüllt automatisch</t>
         </is>
@@ -1767,13 +1812,13 @@
         <v>343.5</v>
       </c>
       <c r="K12" t="n">
-        <v>287559</v>
+        <v>291070</v>
       </c>
       <c r="L12" t="n">
         <v>4164.4</v>
       </c>
       <c r="M12" t="n">
-        <v>69.05</v>
+        <v>69.89</v>
       </c>
       <c r="N12" t="n">
         <v>2</v>
@@ -1787,7 +1832,7 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>3511</v>
       </c>
       <c r="R12" s="48" t="inlineStr">
         <is>
@@ -1796,7 +1841,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-07-22 10:18</t>
+          <t>2026-07-22 18:34</t>
         </is>
       </c>
     </row>
@@ -1836,13 +1881,13 @@
         <v>440.5</v>
       </c>
       <c r="K13" t="n">
-        <v>397312</v>
+        <v>405124</v>
       </c>
       <c r="L13" t="n">
         <v>5591.3</v>
       </c>
       <c r="M13" t="n">
-        <v>71.06</v>
+        <v>72.45999999999999</v>
       </c>
       <c r="N13" t="n">
         <v>2</v>
@@ -1856,7 +1901,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>7812</v>
       </c>
       <c r="R13" s="48" t="inlineStr">
         <is>
@@ -1865,7 +1910,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-07-22 10:18</t>
+          <t>2026-07-22 18:34</t>
         </is>
       </c>
     </row>
@@ -1905,13 +1950,13 @@
         <v>440.5</v>
       </c>
       <c r="K14" t="n">
-        <v>397312</v>
+        <v>405124</v>
       </c>
       <c r="L14" t="n">
         <v>5591.3</v>
       </c>
       <c r="M14" t="n">
-        <v>71.06</v>
+        <v>72.45999999999999</v>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1925,7 +1970,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>7812</v>
       </c>
       <c r="R14" s="48" t="inlineStr">
         <is>
@@ -1934,7 +1979,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-07-22 10:18</t>
+          <t>2026-07-22 18:34</t>
         </is>
       </c>
     </row>
@@ -1974,13 +2019,13 @@
         <v>343.5</v>
       </c>
       <c r="K15" t="n">
-        <v>287559</v>
+        <v>291070</v>
       </c>
       <c r="L15" t="n">
         <v>4164.4</v>
       </c>
       <c r="M15" t="n">
-        <v>69.05</v>
+        <v>69.89</v>
       </c>
       <c r="N15" t="n">
         <v>2</v>
@@ -1994,7 +2039,7 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>3511</v>
       </c>
       <c r="R15" s="48" t="inlineStr">
         <is>
@@ -2003,7 +2048,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-07-22 10:18</t>
+          <t>2026-07-22 18:34</t>
         </is>
       </c>
     </row>
@@ -2028,13 +2073,13 @@
         <v>440.5</v>
       </c>
       <c r="K16" t="n">
-        <v>397312</v>
+        <v>405124</v>
       </c>
       <c r="L16" t="n">
         <v>5591.3</v>
       </c>
       <c r="M16" t="n">
-        <v>71.06</v>
+        <v>72.45999999999999</v>
       </c>
       <c r="N16" t="n">
         <v>1</v>
@@ -2054,10 +2099,209 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-07-22 10:18</t>
-        </is>
-      </c>
-    </row>
+          <t>2026-07-22 18:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19" ht="20" customHeight="1" s="45">
+      <c r="G19" s="63" t="n"/>
+      <c r="H19" s="63" t="n"/>
+      <c r="I19" s="61" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="45">
+      <c r="G20" s="63" t="n"/>
+      <c r="H20" s="63" t="n"/>
+      <c r="I20" s="61" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="45">
+      <c r="G21" s="63" t="n"/>
+      <c r="H21" s="63" t="n"/>
+      <c r="I21" s="62" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="45">
+      <c r="G22" s="63" t="n"/>
+      <c r="H22" s="63" t="n"/>
+      <c r="I22" s="61" t="n"/>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2176,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="45" min="1" max="1"/>
@@ -2299,6 +2543,8 @@
         <v>89.48</v>
       </c>
     </row>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="52" t="inlineStr">
         <is>
@@ -3415,9 +3661,9 @@
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B72:F72"/>
+    <mergeCell ref="B90:F90"/>
     <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B90:F90"/>
-    <mergeCell ref="B72:F72"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B93:F93"/>

</xml_diff>

<commit_message>
Ausgeschiedene THs taggenau in €/h (Zähler+Nenner) — Q2-Tabelle final v3 + Dashboards
_ist_bundle_therapeut(): rollen=Therapeut zählt (Offboarding löscht is_therapeut-Flag),
Geister-Schutz für Inaktive ohne Enddatum. Q2: Laura 308.608 € / 70,32 €/h (15 THs),
Marleen 405.124 € / 69,20 €/h (27 THs) — Stufen unverändert 2/2. Nachdeploy des
gestern abgebrochenen Commits.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1803,22 +1803,22 @@
         <v>8.48</v>
       </c>
       <c r="H12" t="n">
-        <v>5228.9</v>
+        <v>5573.4</v>
       </c>
       <c r="I12" t="n">
-        <v>721</v>
+        <v>819</v>
       </c>
       <c r="J12" t="n">
-        <v>343.5</v>
+        <v>365.5</v>
       </c>
       <c r="K12" t="n">
-        <v>291070</v>
+        <v>308608</v>
       </c>
       <c r="L12" t="n">
-        <v>4164.4</v>
+        <v>4388.9</v>
       </c>
       <c r="M12" t="n">
-        <v>69.89</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="N12" t="n">
         <v>2</v>
@@ -1832,16 +1832,16 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>3511</v>
+        <v>21049</v>
       </c>
       <c r="R12" s="48" t="inlineStr">
         <is>
-          <t>✓ OK</t>
+          <t>⚠️ Diff +7.3 %</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-07-22 18:34</t>
+          <t>2026-07-22 18:52</t>
         </is>
       </c>
     </row>
@@ -1872,22 +1872,22 @@
         <v>7.8</v>
       </c>
       <c r="H13" t="n">
-        <v>7377.3</v>
+        <v>7648.1</v>
       </c>
       <c r="I13" t="n">
         <v>1345.5</v>
       </c>
       <c r="J13" t="n">
-        <v>440.5</v>
+        <v>448.5</v>
       </c>
       <c r="K13" t="n">
         <v>405124</v>
       </c>
       <c r="L13" t="n">
-        <v>5591.3</v>
+        <v>5854.1</v>
       </c>
       <c r="M13" t="n">
-        <v>72.45999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="N13" t="n">
         <v>2</v>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-07-22 18:34</t>
+          <t>2026-07-22 18:52</t>
         </is>
       </c>
     </row>
@@ -1941,22 +1941,22 @@
         <v>9.199999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>7377.3</v>
+        <v>7648.1</v>
       </c>
       <c r="I14" t="n">
         <v>1345.5</v>
       </c>
       <c r="J14" t="n">
-        <v>440.5</v>
+        <v>448.5</v>
       </c>
       <c r="K14" t="n">
         <v>405124</v>
       </c>
       <c r="L14" t="n">
-        <v>5591.3</v>
+        <v>5854.1</v>
       </c>
       <c r="M14" t="n">
-        <v>72.45999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-07-22 18:34</t>
+          <t>2026-07-22 18:52</t>
         </is>
       </c>
     </row>
@@ -2010,22 +2010,22 @@
         <v>9.08</v>
       </c>
       <c r="H15" t="n">
-        <v>5228.9</v>
+        <v>5573.4</v>
       </c>
       <c r="I15" t="n">
-        <v>721</v>
+        <v>819</v>
       </c>
       <c r="J15" t="n">
-        <v>343.5</v>
+        <v>365.5</v>
       </c>
       <c r="K15" t="n">
-        <v>291070</v>
+        <v>308608</v>
       </c>
       <c r="L15" t="n">
-        <v>4164.4</v>
+        <v>4388.9</v>
       </c>
       <c r="M15" t="n">
-        <v>69.89</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="N15" t="n">
         <v>2</v>
@@ -2039,16 +2039,16 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>3511</v>
+        <v>21049</v>
       </c>
       <c r="R15" s="48" t="inlineStr">
         <is>
-          <t>✓ OK</t>
+          <t>⚠️ Diff +7.3 %</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-07-22 18:34</t>
+          <t>2026-07-22 18:52</t>
         </is>
       </c>
     </row>
@@ -2064,22 +2064,22 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>7377.3</v>
+        <v>7648.1</v>
       </c>
       <c r="I16" t="n">
         <v>1345.5</v>
       </c>
       <c r="J16" t="n">
-        <v>440.5</v>
+        <v>448.5</v>
       </c>
       <c r="K16" t="n">
         <v>405124</v>
       </c>
       <c r="L16" t="n">
-        <v>5591.3</v>
+        <v>5854.1</v>
       </c>
       <c r="M16" t="n">
-        <v>72.45999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="N16" t="n">
         <v>1</v>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-07-22 18:34</t>
+          <t>2026-07-22 18:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FINAL: Gehaltsbewertung = Stufe (1) — nur erbrachte Termine, MediFox-deckungsgleich
- compute_quartal: VO-Gebühren + 0,8×geplant aus dem Bewertungs-IST entfernt
  (verschoben die Messlatte um ~8-12 % vs. kalibrierte Schwellen); Vermerk-Blöcke
  in Code, METHODE, ANLEITUNG, SL-Report und Reminder-Mail (n8n) gegen Wiederholung
- Deaktivierungs-Regel aktiv: inaktive THs bis letzter erbrachter Termin (Zähler+Nenner)
- Q2 final: Laura 70,69 €/h (✓ OK, +0,1 % vs. echtem MediFox 291.382), Marleen 69,50
  (✓ plausibel, -8,3 % = 29-Tage-/Deaktivierungs-Abzug vs. 418.775) — Stufen 2/2
- MediFox-Referenzspalte = echte Exportwerte; Status-Logik: nur Modell ÜBER MediFox warnt
- Validierung Stufe (1) H1: alle 5 Standorte ±1,4 %, gesamt +0,3 %

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1797,28 +1797,28 @@
         <v>8.4</v>
       </c>
       <c r="F12" s="38" t="n">
-        <v>287559</v>
+        <v>291382</v>
       </c>
       <c r="G12" t="n">
         <v>8.48</v>
       </c>
       <c r="H12" t="n">
-        <v>5573.4</v>
+        <v>5296.1</v>
       </c>
       <c r="I12" t="n">
-        <v>819</v>
+        <v>805</v>
       </c>
       <c r="J12" t="n">
         <v>365.5</v>
       </c>
       <c r="K12" t="n">
-        <v>308608</v>
+        <v>291653</v>
       </c>
       <c r="L12" t="n">
-        <v>4388.9</v>
+        <v>4125.6</v>
       </c>
       <c r="M12" t="n">
-        <v>70.31999999999999</v>
+        <v>70.69</v>
       </c>
       <c r="N12" t="n">
         <v>2</v>
@@ -1832,16 +1832,16 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>21049</v>
+        <v>271</v>
       </c>
       <c r="R12" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff +7.3 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-07-22 18:52</t>
+          <t>2026-07-23 13:57</t>
         </is>
       </c>
     </row>
@@ -1866,28 +1866,28 @@
         <v>7.8</v>
       </c>
       <c r="F13" s="38" t="n">
-        <v>397312</v>
+        <v>418775</v>
       </c>
       <c r="G13" t="n">
         <v>7.8</v>
       </c>
       <c r="H13" t="n">
-        <v>7648.1</v>
+        <v>7101.8</v>
       </c>
       <c r="I13" t="n">
-        <v>1345.5</v>
+        <v>1145.2</v>
       </c>
       <c r="J13" t="n">
-        <v>448.5</v>
+        <v>428</v>
       </c>
       <c r="K13" t="n">
-        <v>405124</v>
+        <v>384219</v>
       </c>
       <c r="L13" t="n">
-        <v>5854.1</v>
+        <v>5528.5</v>
       </c>
       <c r="M13" t="n">
-        <v>69.2</v>
+        <v>69.5</v>
       </c>
       <c r="N13" t="n">
         <v>2</v>
@@ -1901,16 +1901,16 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>7812</v>
+        <v>-34556</v>
       </c>
       <c r="R13" s="48" t="inlineStr">
         <is>
-          <t>✓ OK</t>
+          <t>✓ plausibel (-8.3 % — 29-Tage-/Deaktivierungs-Abzug)</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-07-22 18:52</t>
+          <t>2026-07-23 13:57</t>
         </is>
       </c>
     </row>
@@ -1935,28 +1935,28 @@
         <v>9.199999999999999</v>
       </c>
       <c r="F14" s="38" t="n">
-        <v>397312</v>
+        <v>418775</v>
       </c>
       <c r="G14" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>7648.1</v>
+        <v>7101.8</v>
       </c>
       <c r="I14" t="n">
-        <v>1345.5</v>
+        <v>1145.2</v>
       </c>
       <c r="J14" t="n">
-        <v>448.5</v>
+        <v>428</v>
       </c>
       <c r="K14" t="n">
-        <v>405124</v>
+        <v>384219</v>
       </c>
       <c r="L14" t="n">
-        <v>5854.1</v>
+        <v>5528.5</v>
       </c>
       <c r="M14" t="n">
-        <v>69.2</v>
+        <v>69.5</v>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1970,16 +1970,16 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>7812</v>
+        <v>-34556</v>
       </c>
       <c r="R14" s="48" t="inlineStr">
         <is>
-          <t>✓ OK</t>
+          <t>✓ plausibel (-8.3 % — 29-Tage-/Deaktivierungs-Abzug)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-07-22 18:52</t>
+          <t>2026-07-23 13:57</t>
         </is>
       </c>
     </row>
@@ -2004,28 +2004,28 @@
         <v>8.9</v>
       </c>
       <c r="F15" s="38" t="n">
-        <v>287559</v>
+        <v>291382</v>
       </c>
       <c r="G15" t="n">
         <v>9.08</v>
       </c>
       <c r="H15" t="n">
-        <v>5573.4</v>
+        <v>5296.1</v>
       </c>
       <c r="I15" t="n">
-        <v>819</v>
+        <v>805</v>
       </c>
       <c r="J15" t="n">
         <v>365.5</v>
       </c>
       <c r="K15" t="n">
-        <v>308608</v>
+        <v>291653</v>
       </c>
       <c r="L15" t="n">
-        <v>4388.9</v>
+        <v>4125.6</v>
       </c>
       <c r="M15" t="n">
-        <v>70.31999999999999</v>
+        <v>70.69</v>
       </c>
       <c r="N15" t="n">
         <v>2</v>
@@ -2039,16 +2039,16 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>21049</v>
+        <v>271</v>
       </c>
       <c r="R15" s="48" t="inlineStr">
         <is>
-          <t>⚠️ Diff +7.3 %</t>
+          <t>✓ OK</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-07-22 18:52</t>
+          <t>2026-07-23 13:57</t>
         </is>
       </c>
     </row>
@@ -2063,23 +2063,26 @@
           <t>Emily</t>
         </is>
       </c>
+      <c r="F16" t="n">
+        <v>418775</v>
+      </c>
       <c r="H16" t="n">
-        <v>7648.1</v>
+        <v>7101.8</v>
       </c>
       <c r="I16" t="n">
-        <v>1345.5</v>
+        <v>1145.2</v>
       </c>
       <c r="J16" t="n">
-        <v>448.5</v>
+        <v>428</v>
       </c>
       <c r="K16" t="n">
-        <v>405124</v>
+        <v>384219</v>
       </c>
       <c r="L16" t="n">
-        <v>5854.1</v>
+        <v>5528.5</v>
       </c>
       <c r="M16" t="n">
-        <v>69.2</v>
+        <v>69.5</v>
       </c>
       <c r="N16" t="n">
         <v>1</v>
@@ -2092,14 +2095,17 @@
           <t>Ja</t>
         </is>
       </c>
+      <c r="Q16" t="n">
+        <v>-34556</v>
+      </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>⏳ Zufriedenheit fehlt</t>
+          <t>✓ plausibel (-8.3 % — 29-Tage-/Deaktivierungs-Abzug)</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-07-22 18:52</t>
+          <t>2026-07-23 13:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Probezeit-Ende innerhalb des Quartals: Gehalt ab Folgetag auf reguläres Modell (Luise/Max ab 01.08.2026 Stufe 2 + Bundle-Zulage); Schienen-Pool (13.08.) mit deployed
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="#,##0\ \€"/>
     <numFmt numFmtId="169" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -219,6 +219,9 @@
       <color rgb="FF666666"/>
       <sz val="16"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -337,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -466,6 +469,7 @@
     <xf numFmtId="3" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1024,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="2"/>
@@ -1314,7 +1318,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="35" t="inlineStr">
         <is>
@@ -1350,39 +1353,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
@@ -1399,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S199"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="1"/>
@@ -2109,8 +2079,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19" ht="20" customHeight="1" s="45">
       <c r="G19" s="63" t="n"/>
       <c r="H19" s="63" t="n"/>
@@ -2131,183 +2099,6 @@
       <c r="H22" s="63" t="n"/>
       <c r="I22" s="61" t="n"/>
     </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2426,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="45" min="1" max="1"/>
@@ -2455,7 +2246,12 @@
       </c>
       <c r="F1" s="16" t="inlineStr">
         <is>
-          <t>€/60min Therapie</t>
+          <t>€/60min Therapie (Basis bis Q2 2026)</t>
+        </is>
+      </c>
+      <c r="G1" s="64" t="inlineStr">
+        <is>
+          <t>€/60min ab Q3 2026 (×1,0411)</t>
         </is>
       </c>
     </row>
@@ -2473,6 +2269,9 @@
       <c r="F2" s="17" t="n">
         <v>61.17</v>
       </c>
+      <c r="G2" t="n">
+        <v>63.68</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="n">
@@ -2488,6 +2287,9 @@
       <c r="F3" s="17" t="n">
         <v>66.54000000000001</v>
       </c>
+      <c r="G3" t="n">
+        <v>69.27</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="n">
@@ -2503,6 +2305,9 @@
       <c r="F4" s="17" t="n">
         <v>72.64</v>
       </c>
+      <c r="G4" t="n">
+        <v>75.63</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="n">
@@ -2518,6 +2323,9 @@
       <c r="F5" s="17" t="n">
         <v>77.28</v>
       </c>
+      <c r="G5" t="n">
+        <v>80.45999999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="n">
@@ -2533,6 +2341,9 @@
       <c r="F6" s="17" t="n">
         <v>84.11</v>
       </c>
+      <c r="G6" t="n">
+        <v>87.56999999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="n">
@@ -2547,6 +2358,9 @@
       </c>
       <c r="F7" s="17" t="n">
         <v>89.48</v>
+      </c>
+      <c r="G7" t="n">
+        <v>93.16</v>
       </c>
     </row>
     <row r="8"/>
@@ -2554,7 +2368,7 @@
     <row r="10">
       <c r="A10" s="52" t="inlineStr">
         <is>
-          <t>Die €/60min-Spalte zeigt Umsatz pro Therapie-Stunde (Bundle-unabhängig, = IST ÷ verfügbare Zeit). Hinweis: Spalte „Leistungsindex" entfiel mit v18 — Stufen-Zuordnung läuft jetzt ausschließlich über €/60min.</t>
+          <t>Die €/60min-Spalte zeigt Umsatz pro Therapie-Stunde (Bundle-unabhängig, = IST ÷ verfügbare Zeit). Hinweis: Spalte „Leistungsindex" entfiel mit v18 — Stufen-Zuordnung läuft jetzt ausschließlich über €/60min. Schwellen-Indexierung (§ 4 Abs. 6): Bei jeder GKV-Satzerhöhung steigen die €/60min-Schwellen mit demselben Faktor — ab Q3 2026 ×1,0411 (Spalte G). Die Q-End-Routine nutzt automatisch die zum Bewertungsquartal gültigen Schwellen (generate.py: stufen_eff). Zufriedenheits-Schwellen und Zulagen-%: unverändert.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Probezeit-Ende: beim Q-Lauf festgelegte Stufe/Anteile gelten festgezurrt bis zur nächsten Q-Bewertung (Spalte Probezeit als Quelle); Q2 nachgetragen: Luise 10 Anteile → 4.042, Max 6 → 2.900
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1369,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S22"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="1"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (bis 31.07.2026; ab 01.08.2026: 4.042 €/Mon = Stufe 2 + 10 Anteile, Teamstand 23.07.2026)</t>
         </is>
       </c>
       <c r="Q14" t="n">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (bis 31.07.2026; ab 01.08.2026: 2.900 €/Mon = Stufe 2 + 6 Anteile, Teamstand 23.07.2026)</t>
         </is>
       </c>
       <c r="Q15" t="n">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (bis 31.12.2026)</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -2079,6 +2079,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19" ht="20" customHeight="1" s="45">
       <c r="G19" s="63" t="n"/>
       <c r="H19" s="63" t="n"/>
@@ -2099,6 +2101,13 @@
       <c r="H22" s="63" t="n"/>
       <c r="I22" s="61" t="n"/>
     </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
@@ -2363,8 +2372,6 @@
         <v>93.16</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Bundle-Zulage je Quartal fest (Valentin 18.08.2026): Anteile beim Q-Lauf in Spalte 20 der Q-Zeile, gelten bis zur nächsten Bewertung; Q1/Q2 nachgetragen (Q3: Laura 7, Max 6, Marleen 10, Luise 10, Emily 0); Dashboards neu
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -1369,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="45" min="1" max="1"/>
@@ -1386,6 +1386,7 @@
     <col width="16" customWidth="1" style="45" min="17" max="17"/>
     <col width="24" customWidth="1" style="45" min="18" max="18"/>
     <col width="18" customWidth="1" style="45" min="19" max="19"/>
+    <col width="14" customWidth="1" style="45" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1" s="45">
@@ -1505,6 +1506,11 @@
           <t>Berechnet am</t>
         </is>
       </c>
+      <c r="T7" s="37" t="inlineStr">
+        <is>
+          <t>Bundle-Anteile (fix)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1572,6 +1578,9 @@
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
       </c>
+      <c r="T8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1638,6 +1647,9 @@
         <is>
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
+      </c>
+      <c r="T9" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1690,6 +1702,9 @@
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
       </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1745,6 +1760,9 @@
           <t>2026-03-31 (Excel-Bestand, alte Methode)</t>
         </is>
       </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1814,6 +1832,9 @@
           <t>2026-07-23 13:57</t>
         </is>
       </c>
+      <c r="T12" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1883,6 +1904,9 @@
           <t>2026-07-23 13:57</t>
         </is>
       </c>
+      <c r="T13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1952,6 +1976,9 @@
           <t>2026-07-23 13:57</t>
         </is>
       </c>
+      <c r="T14" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2021,6 +2048,9 @@
           <t>2026-07-23 13:57</t>
         </is>
       </c>
+      <c r="T15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2077,6 +2107,9 @@
         <is>
           <t>2026-07-23 13:57</t>
         </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17"/>
@@ -2101,13 +2134,6 @@
       <c r="H22" s="63" t="n"/>
       <c r="I22" s="61" t="n"/>
     </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>

</xml_diff>

<commit_message>
PM-Stammdaten: Anna (Spandau/Mitte, seit 01.08.2026) im Excel + Q2-Basiszeile, Dashboard erzeugt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqbWVytn6s6zGpM6C5kh5F
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -21,13 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0\ \€"/>
     <numFmt numFmtId="169" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -1118,7 +1119,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="51" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="D6" s="51" t="n">
         <v>45000</v>
@@ -1131,7 +1132,7 @@
       </c>
       <c r="G6" s="51" t="inlineStr">
         <is>
-          <t>Laura, Max</t>
+          <t>Laura, Max, Anna</t>
         </is>
       </c>
       <c r="H6" s="51" t="inlineStr">
@@ -1242,7 +1243,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="51" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="D9" s="51" t="n">
         <v>40000</v>
@@ -1259,7 +1260,7 @@
       </c>
       <c r="G9" s="51" t="inlineStr">
         <is>
-          <t>Laura, Max</t>
+          <t>Laura, Max, Anna</t>
         </is>
       </c>
       <c r="H9" s="51" t="inlineStr">
@@ -1315,6 +1316,48 @@
         </is>
       </c>
       <c r="J10" s="51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1" s="45">
+      <c r="A11" s="51" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="B11" s="51" t="n">
+        <v>40</v>
+      </c>
+      <c r="C11" s="51" t="n">
+        <v>110</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E11" s="43" t="n">
+        <v>46235</v>
+      </c>
+      <c r="F11" s="51" t="inlineStr">
+        <is>
+          <t>Spandau, Mitte</t>
+        </is>
+      </c>
+      <c r="G11" s="51" t="inlineStr">
+        <is>
+          <t>Laura, Max, Anna</t>
+        </is>
+      </c>
+      <c r="H11" s="51" t="inlineStr">
+        <is>
+          <t>#795548</t>
+        </is>
+      </c>
+      <c r="I11" s="51" t="inlineStr">
+        <is>
+          <t>77f8ad35bf3130d63658dc9dbf5c5898</t>
+        </is>
+      </c>
+      <c r="J11" s="51" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2052,7 +2095,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" s="45">
       <c r="A16" t="inlineStr">
         <is>
           <t>Q2 2026</t>
@@ -2112,8 +2155,66 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
+    <row r="17" s="45">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>291382</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5296.1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>805</v>
+      </c>
+      <c r="J17" t="n">
+        <v>365.5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>291653</v>
+      </c>
+      <c r="L17" t="n">
+        <v>4125.6</v>
+      </c>
+      <c r="M17" t="n">
+        <v>70.69</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Ja (bis 31.01.2027)</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>271</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-09-09 (Stammdaten nachgetragen, Bundle-Werte = Laura Q2)</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="19" ht="20" customHeight="1" s="45">
       <c r="G19" s="63" t="n"/>
       <c r="H19" s="63" t="n"/>

</xml_diff>

<commit_message>
PM-Stammdaten: Max 40 h seit 01.09.2026 (PM-Std Bundle 120); Dashboards neu erzeugt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqbWVytn6s6zGpM6C5kh5F
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell.xlsx
+++ b/generator/PM_Gehaltsmodell.xlsx
@@ -21,14 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0\ \€"/>
     <numFmt numFmtId="169" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -1119,7 +1118,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="51" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D6" s="51" t="n">
         <v>45000</v>
@@ -1240,10 +1239,10 @@
         </is>
       </c>
       <c r="B9" s="51" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C9" s="51" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D9" s="51" t="n">
         <v>40000</v>
@@ -1329,7 +1328,7 @@
         <v>40</v>
       </c>
       <c r="C11" s="51" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D11" s="51" t="n">
         <v>40000</v>

</xml_diff>